<commit_message>
Auto: PA-jobb uppdatering latest
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋  Lediga PA-jobb – MANLIGA KUNDER – Uppsala  |  ✅ UPPDATERAD 13 mars 2026  |  20 aktiva jobb  |  🆕 1 ny efter 9 mar: Kura Omsorg Heby (man, pub 10 mars #30724355)  |  Pub-datum verifierade Assistanskoll/Platsbanken</t>
+          <t>📋  Lediga PA-jobb – MANLIGA KUNDER – Uppsala  |  ✅ UPPDATERAD 2026-03-19  |  35 nya tillkomna  |  0 utgångna borttagna</t>
         </is>
       </c>
     </row>
@@ -3218,7 +3218,7 @@
       <c r="M4" s="104" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="143" t="inlineStr">
+      <c r="A5" s="161" t="inlineStr">
         <is>
           <t>⭐⭐⭐  PERFEKT MATCH — Manlig kund, helg/kväll, nära Gunsta  |  Uppdaterad 13 mars 2026</t>
         </is>
@@ -4631,24 +4631,2477 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="35" customHeight="1">
-      <c r="A28" s="135" t="inlineStr">
+    <row r="28" ht="55" customHeight="1">
+      <c r="A28" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B28" s="133" t="inlineStr">
+        <is>
+          <t>Vi söker nu personlig assistent till kund som bor i Östervåla</t>
+        </is>
+      </c>
+      <c r="C28" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D28" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E28" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F28" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G28" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H28" s="158" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="I28" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J28" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K28" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L28" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Deadline före semester – sök INNAN 8 juni.</t>
+        </is>
+      </c>
+      <c r="M28" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-19
+Platsbanken #30770793</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="135" t="inlineStr">
         <is>
           <t>📌 BORTTAGNA: SAAND Uppsala (dead 15 mar) | Särnmark ung man 24år (dead 11 mar) | Humana 19-årig kille (dead 27 feb) | IT-kille Särnmark (dead 13 feb)  —  🆕 EFTER 9 MAR: Kura Omsorg Heby man #30724355 (pub 10 mars)  —  KÄLLOR: Platsbanken · Assistanskoll · Indeed · ledigajobb.se · vakanser.se</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1"/>
+    <row r="30" ht="55" customHeight="1">
+      <c r="A30" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B30" s="133" t="inlineStr">
+        <is>
+          <t>Vi söker nu personlig assistent till kund som bor i Östervåla</t>
+        </is>
+      </c>
+      <c r="C30" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D30" s="157" t="inlineStr">
+        <is>
+          <t>Tierp</t>
+        </is>
+      </c>
+      <c r="E30" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F30" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G30" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H30" s="158" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="I30" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J30" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K30" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L30" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Deadline före semester – sök INNAN 8 juni.</t>
+        </is>
+      </c>
+      <c r="M30" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-19
+Platsbanken #30770710</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32" ht="55" customHeight="1">
+      <c r="A32" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B32" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent till man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C32" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D32" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E32" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F32" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G32" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H32" s="158" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I32" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J32" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K32" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L32" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst. = ta inga pass 8 jun–3 jul.</t>
+        </is>
+      </c>
+      <c r="M32" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-19
+Platsbanken #30769628</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="55" customHeight="1">
+      <c r="A34" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B34" s="133" t="inlineStr">
+        <is>
+          <t>Sommarjobb som personlig assistent (Tierp med omnejd)</t>
+        </is>
+      </c>
+      <c r="C34" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D34" s="157" t="inlineStr">
+        <is>
+          <t>Tierp med omnejd) 5 arbetsplatser, deltid ,
+ 11 dagar - upp till 3 månader,
+ varaktighet: sommarjobb / feriejobb Vivida Assistans AB (Tierp</t>
+        </is>
+      </c>
+      <c r="E34" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F34" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G34" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H34" s="158" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="I34" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J34" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K34" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L34" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat = troligen behövs under din semester (8 jun–3 jul).</t>
+        </is>
+      </c>
+      <c r="M34" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-16
+Platsbanken #30751923</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="55" customHeight="1">
+      <c r="A36" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B36" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till aktiv ung man i Knivsta</t>
+        </is>
+      </c>
+      <c r="C36" s="145" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D36" s="145" t="inlineStr">
+        <is>
+          <t>Knivsta</t>
+        </is>
+      </c>
+      <c r="E36" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F36" s="145" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G36" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H36" s="146" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="I36" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J36" s="145" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K36" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L36" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Deadline före semester – sök INNAN 8 juni.</t>
+        </is>
+      </c>
+      <c r="M36" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-16
+Platsbanken #30751040</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="55" customHeight="1">
+      <c r="A38" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B38" s="133" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C38" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D38" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E38" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F38" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G38" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H38" s="158" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I38" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J38" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K38" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L38" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+6 mån+ – diskutera semester vid intervju.</t>
+        </is>
+      </c>
+      <c r="M38" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-16
+Platsbanken #30749853</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="55" customHeight="1">
+      <c r="A40" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B40" s="133" t="inlineStr">
+        <is>
+          <t>Meningsfullt PA-jobb – personlig assistent sökes till barn i Björklinge!</t>
+        </is>
+      </c>
+      <c r="C40" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D40" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E40" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F40" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G40" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H40" s="158" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="I40" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J40" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K40" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L40" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare = semester förhandlas normalt.</t>
+        </is>
+      </c>
+      <c r="M40" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-13
+Platsbanken #30744655</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="55" customHeight="1">
+      <c r="A42" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B42" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent - Deltidstjänst Habo (Körkort är ett krav)</t>
+        </is>
+      </c>
+      <c r="C42" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D42" s="152" t="inlineStr">
+        <is>
+          <t>Habo</t>
+        </is>
+      </c>
+      <c r="E42" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F42" s="152" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G42" s="153" t="inlineStr">
+        <is>
+          <t>✅ KRÄVS</t>
+        </is>
+      </c>
+      <c r="H42" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="I42" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J42" s="152" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K42" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L42" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst. = ta inga pass 8 jun–3 jul.</t>
+        </is>
+      </c>
+      <c r="M42" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-12
+Platsbanken #30700718</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="55" customHeight="1">
+      <c r="A44" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B44" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent för timvikariat sökes till man i Heby</t>
+        </is>
+      </c>
+      <c r="C44" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D44" s="157" t="inlineStr">
+        <is>
+          <t>Heby</t>
+        </is>
+      </c>
+      <c r="E44" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F44" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G44" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H44" s="158" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="I44" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J44" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K44" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L44" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst. = ta inga pass 8 jun–3 jul.</t>
+        </is>
+      </c>
+      <c r="M44" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-10
+Platsbanken #30724355</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="55" customHeight="1">
+      <c r="A46" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B46" s="123" t="inlineStr">
+        <is>
+          <t>Vi söker personliga assistenter till ett barn i Storvreta</t>
+        </is>
+      </c>
+      <c r="C46" s="145" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D46" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E46" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F46" s="145" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G46" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H46" s="146" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="I46" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J46" s="145" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K46" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L46" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare = semester förhandlas normalt.</t>
+        </is>
+      </c>
+      <c r="M46" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-09
+Platsbanken #30717131</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="55" customHeight="1">
+      <c r="A48" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B48" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent- Sommarvikariat</t>
+        </is>
+      </c>
+      <c r="C48" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D48" s="157" t="inlineStr">
+        <is>
+          <t>Heby</t>
+        </is>
+      </c>
+      <c r="E48" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F48" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G48" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H48" s="158" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="I48" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J48" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K48" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L48" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat = troligen behövs under din semester (8 jun–3 jul).</t>
+        </is>
+      </c>
+      <c r="M48" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-09
+Platsbanken #30715191</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="55" customHeight="1">
+      <c r="A50" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B50" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent på deltid, varannan helg (25%)</t>
+        </is>
+      </c>
+      <c r="C50" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D50" s="152" t="inlineStr">
+        <is>
+          <t>25%) Deltid ,
+ tills vidare,
+ varaktighet: vanlig anställning Akut bemanning och rekrytering Assistansakuten i (Uppsala</t>
+        </is>
+      </c>
+      <c r="E50" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F50" s="152" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G50" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H50" s="153" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="I50" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J50" s="152" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K50" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L50" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare = semester förhandlas normalt.</t>
+        </is>
+      </c>
+      <c r="M50" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-09
+Platsbanken #30714687</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="55" customHeight="1">
+      <c r="A52" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B52" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent- Uppsala</t>
+        </is>
+      </c>
+      <c r="C52" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D52" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E52" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F52" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G52" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H52" s="158" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="I52" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J52" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K52" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L52" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst. = ta inga pass 8 jun–3 jul.</t>
+        </is>
+      </c>
+      <c r="M52" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+Platsbanken #30703817</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="55" customHeight="1">
+      <c r="A54" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B54" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent till en man i Enköping</t>
+        </is>
+      </c>
+      <c r="C54" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D54" s="157" t="inlineStr">
+        <is>
+          <t>Enköping</t>
+        </is>
+      </c>
+      <c r="E54" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F54" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G54" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H54" s="158" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="I54" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J54" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K54" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L54" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare = semester förhandlas normalt.</t>
+        </is>
+      </c>
+      <c r="M54" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-04
+Platsbanken #30693340</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="55" customHeight="1">
+      <c r="A56" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B56" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent</t>
+        </is>
+      </c>
+      <c r="C56" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D56" s="157" t="inlineStr">
+        <is>
+          <t>Habo</t>
+        </is>
+      </c>
+      <c r="E56" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F56" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G56" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H56" s="158" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="I56" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J56" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K56" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L56" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare = semester förhandlas normalt.</t>
+        </is>
+      </c>
+      <c r="M56" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-03
+Platsbanken #30687951</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="55" customHeight="1">
+      <c r="A58" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B58" s="133" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C58" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D58" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E58" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F58" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G58" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H58" s="158" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I58" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J58" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K58" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L58" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare = semester förhandlas normalt.</t>
+        </is>
+      </c>
+      <c r="M58" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-03
+Platsbanken #30687806</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="55" customHeight="1">
+      <c r="A60" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B60" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent, timanställning/sommarpersonal, väster om Uppsala</t>
+        </is>
+      </c>
+      <c r="C60" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D60" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E60" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F60" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G60" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H60" s="158" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="I60" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J60" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K60" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L60" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat = troligen behövs under din semester (8 jun–3 jul).</t>
+        </is>
+      </c>
+      <c r="M60" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-03
+Platsbanken #30686751</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="55" customHeight="1">
+      <c r="A62" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B62" s="133" t="inlineStr">
+        <is>
+          <t>Personliga assistenter sökes till kille utanför Uppsala</t>
+        </is>
+      </c>
+      <c r="C62" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D62" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E62" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F62" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G62" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H62" s="158" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="I62" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J62" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K62" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L62" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare = semester förhandlas normalt.</t>
+        </is>
+      </c>
+      <c r="M62" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-26
+Platsbanken #30667617</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="55" customHeight="1">
+      <c r="A64" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B64" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C64" s="145" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D64" s="145" t="inlineStr">
+        <is>
+          <t>Tierp</t>
+        </is>
+      </c>
+      <c r="E64" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F64" s="145" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G64" s="146" t="inlineStr">
+        <is>
+          <t>✅ KRÄVS</t>
+        </is>
+      </c>
+      <c r="H64" s="146" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I64" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J64" s="145" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K64" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L64" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Deadline före semester – sök INNAN 8 juni.</t>
+        </is>
+      </c>
+      <c r="M64" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-26
+Platsbanken #30666709</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="55" customHeight="1">
+      <c r="A66" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B66" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C66" s="145" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D66" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E66" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F66" s="145" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G66" s="146" t="inlineStr">
+        <is>
+          <t>✅ KRÄVS</t>
+        </is>
+      </c>
+      <c r="H66" s="146" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I66" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J66" s="145" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K66" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L66" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Deadline före semester – sök INNAN 8 juni.</t>
+        </is>
+      </c>
+      <c r="M66" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-26
+Platsbanken #30666685</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="55" customHeight="1">
+      <c r="A68" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B68" s="133" t="inlineStr">
+        <is>
+          <t>Vi söker nu personliga assistenter till kund som bor i Östervåla</t>
+        </is>
+      </c>
+      <c r="C68" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D68" s="157" t="inlineStr">
+        <is>
+          <t>Heby</t>
+        </is>
+      </c>
+      <c r="E68" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F68" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G68" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H68" s="158" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="I68" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J68" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K68" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L68" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Deadline före semester – sök INNAN 8 juni.</t>
+        </is>
+      </c>
+      <c r="M68" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-24
+Platsbanken #30654789</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="55" customHeight="1">
+      <c r="A70" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B70" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent, behovsvikarie</t>
+        </is>
+      </c>
+      <c r="C70" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D70" s="157" t="inlineStr">
+        <is>
+          <t>Tierp</t>
+        </is>
+      </c>
+      <c r="E70" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F70" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G70" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H70" s="158" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="I70" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J70" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K70" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L70" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst. = ta inga pass 8 jun–3 jul.</t>
+        </is>
+      </c>
+      <c r="M70" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+Platsbanken #30652160</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="55" customHeight="1">
+      <c r="A72" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B72" s="133" t="inlineStr">
+        <is>
+          <t>Sommarvikarie - Personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C72" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D72" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E72" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F72" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G72" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H72" s="158" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I72" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J72" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K72" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L72" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat = troligen behövs under din semester (8 jun–3 jul).</t>
+        </is>
+      </c>
+      <c r="M72" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+Platsbanken #30651918</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="55" customHeight="1">
+      <c r="A74" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B74" s="133" t="inlineStr">
+        <is>
+          <t>Sommarvikarie - Personlig assistent i Håbo</t>
+        </is>
+      </c>
+      <c r="C74" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D74" s="157" t="inlineStr">
+        <is>
+          <t>Håbo</t>
+        </is>
+      </c>
+      <c r="E74" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F74" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G74" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H74" s="158" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I74" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J74" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K74" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L74" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat = troligen behövs under din semester (8 jun–3 jul).</t>
+        </is>
+      </c>
+      <c r="M74" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+Platsbanken #30651895</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="55" customHeight="1">
+      <c r="A76" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B76" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C76" s="145" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D76" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E76" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F76" s="145" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G76" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H76" s="146" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="I76" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J76" s="145" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K76" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L76" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Deadline före semester – sök INNAN 8 juni.</t>
+        </is>
+      </c>
+      <c r="M76" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+Platsbanken #30647293</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="55" customHeight="1">
+      <c r="A78" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B78" s="133" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C78" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D78" s="157" t="inlineStr">
+        <is>
+          <t>Enköping</t>
+        </is>
+      </c>
+      <c r="E78" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F78" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G78" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H78" s="158" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="I78" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J78" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K78" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L78" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Deadline före semester – sök INNAN 8 juni.</t>
+        </is>
+      </c>
+      <c r="M78" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-20
+Platsbanken #30638977</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="55" customHeight="1">
+      <c r="A80" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B80" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent åt kille i Knivsta</t>
+        </is>
+      </c>
+      <c r="C80" s="145" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D80" s="145" t="inlineStr">
+        <is>
+          <t>Knivsta</t>
+        </is>
+      </c>
+      <c r="E80" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F80" s="145" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G80" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H80" s="146" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="I80" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J80" s="145" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K80" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L80" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare = semester förhandlas normalt.</t>
+        </is>
+      </c>
+      <c r="M80" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-16
+Platsbanken #30616398</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="55" customHeight="1">
+      <c r="A82" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B82" s="133" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C82" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D82" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E82" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F82" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G82" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H82" s="158" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="I82" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J82" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K82" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L82" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat = troligen behövs under din semester (8 jun–3 jul).</t>
+        </is>
+      </c>
+      <c r="M82" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-12
+Platsbanken #30603880</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="55" customHeight="1">
+      <c r="A84" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B84" s="133" t="inlineStr">
+        <is>
+          <t>Sommarvikariat som personlig assistent - Uppsala</t>
+        </is>
+      </c>
+      <c r="C84" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D84" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E84" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F84" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G84" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H84" s="158" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="I84" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J84" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K84" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L84" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat = troligen behövs under din semester (8 jun–3 jul).</t>
+        </is>
+      </c>
+      <c r="M84" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-03
+Platsbanken #30554923</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="55" customHeight="1">
+      <c r="A86" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B86" s="133" t="inlineStr">
+        <is>
+          <t>Sommarjobba som personlig assistent i området Habo och Mullsjö</t>
+        </is>
+      </c>
+      <c r="C86" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D86" s="157" t="inlineStr">
+        <is>
+          <t>Habo</t>
+        </is>
+      </c>
+      <c r="E86" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F86" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G86" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H86" s="158" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="I86" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J86" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K86" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L86" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat = troligen behövs under din semester (8 jun–3 jul).</t>
+        </is>
+      </c>
+      <c r="M86" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-01-15
+Platsbanken #30477728</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="55" customHeight="1">
+      <c r="A88" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B88" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent åt man i Enköping</t>
+        </is>
+      </c>
+      <c r="C88" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D88" s="157" t="inlineStr">
+        <is>
+          <t>Enköping</t>
+        </is>
+      </c>
+      <c r="E88" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F88" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G88" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H88" s="158" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="I88" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J88" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K88" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L88" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Deadline före semester – sök INNAN 8 juni.</t>
+        </is>
+      </c>
+      <c r="M88" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-01-08
+Platsbanken #30445221</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="55" customHeight="1">
+      <c r="A90" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B90" s="133" t="inlineStr">
+        <is>
+          <t>Assistent sökes till glad och aktiv man i Gimo</t>
+        </is>
+      </c>
+      <c r="C90" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D90" s="157" t="inlineStr">
+        <is>
+          <t>Östhammar</t>
+        </is>
+      </c>
+      <c r="E90" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F90" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G90" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H90" s="158" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="I90" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J90" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K90" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L90" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare = semester förhandlas normalt.</t>
+        </is>
+      </c>
+      <c r="M90" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-01-07
+Platsbanken #30441435</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="55" customHeight="1">
+      <c r="A92" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B92" s="133" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C92" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D92" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E92" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F92" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G92" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H92" s="158" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="I92" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J92" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K92" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L92" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Deadline före semester – sök INNAN 8 juni.</t>
+        </is>
+      </c>
+      <c r="M92" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-01-02
+Platsbanken #30430160</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="55" customHeight="1">
+      <c r="A94" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B94" s="133" t="inlineStr">
+        <is>
+          <t>Vi söker nu personliga assistenter till kunder som bor i Uppland.</t>
+        </is>
+      </c>
+      <c r="C94" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D94" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E94" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F94" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G94" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H94" s="158" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="I94" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J94" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K94" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L94" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Deadline före semester – sök INNAN 8 juni.</t>
+        </is>
+      </c>
+      <c r="M94" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2025-11-19
+Platsbanken #30280822</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="55" customHeight="1">
+      <c r="A96" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B96" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent</t>
+        </is>
+      </c>
+      <c r="C96" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D96" s="157" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E96" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F96" s="157" t="inlineStr">
+        <is>
+          <t>🗓️ Kontrollera annons</t>
+        </is>
+      </c>
+      <c r="G96" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H96" s="158" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I96" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J96" s="157" t="inlineStr">
+        <is>
+          <t>Ny annons! Kolla detaljer på Platsbanken.</t>
+        </is>
+      </c>
+      <c r="K96" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L96" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare = semester förhandlas normalt.</t>
+        </is>
+      </c>
+      <c r="M96" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2025-11-18
+Platsbanken #30277802</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="7">
     <mergeCell ref="A29:L29"/>
+    <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A1:M1"/>
     <mergeCell ref="A12:M12"/>
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A24:M24"/>
-    <mergeCell ref="A28:M28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId1"/>
@@ -4672,6 +7125,41 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B58" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B66" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B82" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B90" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B94" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B96" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-03-20
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M96"/>
+  <dimension ref="A1:M109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋  Lediga PA-jobb – MANLIGA KUNDER – Uppsala  |  ✅ UPPDATERAD 2026-03-19  |  Radie: &lt;50 km från Gunsta  |  0 nya tillkomna  |  25 utgångna borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-20 · 3 källor · Radie &lt;50 km · 13 nya · 10 borttagna</t>
         </is>
       </c>
     </row>
@@ -7122,6 +7122,889 @@
           <t>🆕 NYTT
 2025-11-18
 Platsbanken #30277802</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="55" customHeight="1">
+      <c r="A97" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B97" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C97" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D97" s="145" t="inlineStr">
+        <is>
+          <t>Tierp</t>
+        </is>
+      </c>
+      <c r="E97" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F97" s="145" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G97" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H97" s="146" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I97" s="146" t="inlineStr">
+        <is>
+          <t>~42 km</t>
+        </is>
+      </c>
+      <c r="J97" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K97" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L97" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Sök INNAN semestern.</t>
+        </is>
+      </c>
+      <c r="M97" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-26
+🏛️ Platsbanken #30666709</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="55" customHeight="1">
+      <c r="A98" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B98" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C98" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D98" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E98" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F98" s="145" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G98" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H98" s="146" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I98" s="146" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J98" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K98" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L98" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Sök INNAN semestern.</t>
+        </is>
+      </c>
+      <c r="M98" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-26
+🏛️ Platsbanken #30666685</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="55" customHeight="1">
+      <c r="A99" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B99" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C99" s="145" t="inlineStr"/>
+      <c r="D99" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E99" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F99" s="145" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G99" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H99" s="146" t="inlineStr"/>
+      <c r="I99" s="146" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J99" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K99" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L99" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M99" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="55" customHeight="1">
+      <c r="A100" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B100" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C100" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D100" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E100" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F100" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G100" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H100" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I100" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J100" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K100" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L100" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M100" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-19
+🏛️ Platsbanken #30769628</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="55" customHeight="1">
+      <c r="A101" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B101" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till aktiv ung man i Knivsta</t>
+        </is>
+      </c>
+      <c r="C101" s="152" t="inlineStr">
+        <is>
+          <t>Särnmark Assistans AB</t>
+        </is>
+      </c>
+      <c r="D101" s="152" t="inlineStr">
+        <is>
+          <t>Knivsta</t>
+        </is>
+      </c>
+      <c r="E101" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F101" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G101" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H101" s="153" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="I101" s="153" t="inlineStr">
+        <is>
+          <t>~29 km</t>
+        </is>
+      </c>
+      <c r="J101" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K101" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L101" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Sök INNAN semestern.</t>
+        </is>
+      </c>
+      <c r="M101" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-16
+🏛️ Platsbanken #30751040</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="55" customHeight="1">
+      <c r="A102" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B102" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C102" s="152" t="inlineStr">
+        <is>
+          <t>Inkludera Assistans AB</t>
+        </is>
+      </c>
+      <c r="D102" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E102" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F102" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G102" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H102" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I102" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J102" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K102" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L102" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M102" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-03
+🏛️ Platsbanken #30687806</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="55" customHeight="1">
+      <c r="A103" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B103" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter sökes till kille utanför Uppsala</t>
+        </is>
+      </c>
+      <c r="C103" s="152" t="inlineStr">
+        <is>
+          <t>Glaucus Assistans AB</t>
+        </is>
+      </c>
+      <c r="D103" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E103" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F103" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G103" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H103" s="153" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="I103" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J103" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K103" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L103" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M103" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-26
+🏛️ Platsbanken #30667617</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="55" customHeight="1">
+      <c r="A104" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B104" s="129" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C104" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D104" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E104" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F104" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G104" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H104" s="153" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="I104" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J104" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K104" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L104" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Sök INNAN semestern.</t>
+        </is>
+      </c>
+      <c r="M104" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🏛️ Platsbanken #30647293</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="55" customHeight="1">
+      <c r="A105" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B105" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent åt kille i Knivsta</t>
+        </is>
+      </c>
+      <c r="C105" s="152" t="inlineStr">
+        <is>
+          <t>Särnmark Assistans AB</t>
+        </is>
+      </c>
+      <c r="D105" s="152" t="inlineStr">
+        <is>
+          <t>Knivsta</t>
+        </is>
+      </c>
+      <c r="E105" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F105" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G105" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H105" s="153" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="I105" s="153" t="inlineStr">
+        <is>
+          <t>~29 km</t>
+        </is>
+      </c>
+      <c r="J105" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K105" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L105" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M105" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-16
+🏛️ Platsbanken #30616398</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="55" customHeight="1">
+      <c r="A106" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B106" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C106" s="152" t="inlineStr"/>
+      <c r="D106" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E106" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F106" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G106" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H106" s="153" t="inlineStr"/>
+      <c r="I106" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J106" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K106" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L106" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M106" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="55" customHeight="1">
+      <c r="A107" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B107" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter sökes till kille utanför Uppsala</t>
+        </is>
+      </c>
+      <c r="C107" s="152" t="inlineStr"/>
+      <c r="D107" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E107" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F107" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G107" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H107" s="153" t="inlineStr"/>
+      <c r="I107" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J107" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K107" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L107" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M107" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="55" customHeight="1">
+      <c r="A108" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B108" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent för timvikariat sökes till man i Heby</t>
+        </is>
+      </c>
+      <c r="C108" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D108" s="157" t="inlineStr">
+        <is>
+          <t>Heby</t>
+        </is>
+      </c>
+      <c r="E108" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F108" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G108" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H108" s="158" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="I108" s="158" t="inlineStr">
+        <is>
+          <t>~49 km</t>
+        </is>
+      </c>
+      <c r="J108" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K108" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L108" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M108" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-10
+🏛️ Platsbanken #30724355</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="55" customHeight="1">
+      <c r="A109" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B109" s="133" t="inlineStr">
+        <is>
+          <t>Assistent sökes till glad och aktiv man i Gimo</t>
+        </is>
+      </c>
+      <c r="C109" s="157" t="inlineStr">
+        <is>
+          <t>Vår Omtanke Sverige AB</t>
+        </is>
+      </c>
+      <c r="D109" s="157" t="inlineStr">
+        <is>
+          <t>Östhammar</t>
+        </is>
+      </c>
+      <c r="E109" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F109" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G109" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H109" s="158" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="I109" s="158" t="inlineStr">
+        <is>
+          <t>~45 km</t>
+        </is>
+      </c>
+      <c r="J109" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K109" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L109" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M109" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-01-07
+🏛️ Platsbanken #30441435</t>
         </is>
       </c>
     </row>
@@ -7192,6 +8075,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B94" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B96" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B97" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B99" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B100" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B101" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B105" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B106" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B107" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B108" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B109" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-03-21
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M109"/>
+  <dimension ref="A1:M115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-20 · 3 källor · Radie &lt;50 km · 13 nya · 10 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-21 · 3 källor · Radie &lt;50 km · 6 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -8005,6 +8005,399 @@
           <t>🆕 NYTT
 2026-01-07
 🏛️ Platsbanken #30441435</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="55" customHeight="1">
+      <c r="A110" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B110" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C110" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D110" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E110" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F110" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G110" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H110" s="153" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="I110" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J110" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K110" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L110" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Sök INNAN semestern.</t>
+        </is>
+      </c>
+      <c r="M110" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-20
+🏛️ Platsbanken #30779004</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="55" customHeight="1">
+      <c r="A111" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B111" s="129" t="inlineStr">
+        <is>
+          <t>Assistent sökes till 4-årig pojke i Uppsala</t>
+        </is>
+      </c>
+      <c r="C111" s="152" t="inlineStr">
+        <is>
+          <t>Aberia AB</t>
+        </is>
+      </c>
+      <c r="D111" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E111" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F111" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G111" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H111" s="153" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="I111" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J111" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K111" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L111" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M111" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-20
+🏛️ Platsbanken #30776985</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="55" customHeight="1">
+      <c r="A112" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B112" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C112" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D112" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E112" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F112" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G112" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H112" s="153" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I112" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J112" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K112" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L112" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M112" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-20
+🏛️ Platsbanken #30775425</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="55" customHeight="1">
+      <c r="A113" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B113" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C113" s="152" t="inlineStr"/>
+      <c r="D113" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E113" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F113" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G113" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H113" s="153" t="inlineStr"/>
+      <c r="I113" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J113" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K113" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L113" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M113" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="55" customHeight="1">
+      <c r="A114" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B114" s="129" t="inlineStr">
+        <is>
+          <t>Assistent sökes till 4-årig pojke i Uppsala</t>
+        </is>
+      </c>
+      <c r="C114" s="152" t="inlineStr"/>
+      <c r="D114" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E114" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F114" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G114" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H114" s="153" t="inlineStr"/>
+      <c r="I114" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J114" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K114" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L114" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M114" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="55" customHeight="1">
+      <c r="A115" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B115" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C115" s="152" t="inlineStr"/>
+      <c r="D115" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E115" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F115" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G115" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H115" s="153" t="inlineStr"/>
+      <c r="I115" s="153" t="inlineStr">
+        <is>
+          <t>~16 km</t>
+        </is>
+      </c>
+      <c r="J115" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K115" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L115" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M115" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -8088,6 +8481,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B107" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B108" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B109" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B112" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B113" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" r:id="rId75"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-03-25
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M115"/>
+  <dimension ref="A1:M116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-21 · 3 källor · Radie &lt;50 km · 0 nya · 6 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-25 · 3 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -8398,6 +8398,76 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="55" customHeight="1">
+      <c r="A116" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B116" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till aktiv man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C116" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D116" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E116" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F116" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G116" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H116" s="153" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="I116" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J116" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K116" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L116" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M116" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-24
+🏛️ Platsbanken #30791374</t>
         </is>
       </c>
     </row>
@@ -8487,6 +8557,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B113" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B116" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-03-26
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M116"/>
+  <dimension ref="A1:M117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-25 · 3 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-26 · 3 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -8468,6 +8468,76 @@
           <t>🆕 NYTT
 2026-03-24
 🏛️ Platsbanken #30791374</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="55" customHeight="1">
+      <c r="A117" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B117" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till kreativ 19-årig kille i Uppsala/Norrtälje</t>
+        </is>
+      </c>
+      <c r="C117" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D117" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E117" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F117" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G117" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H117" s="153" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="I117" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J117" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K117" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L117" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M117" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-25
+🏛️ Platsbanken #30798017</t>
         </is>
       </c>
     </row>
@@ -8558,6 +8628,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B116" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B117" r:id="rId77"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-03-27
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M117"/>
+  <dimension ref="A1:M118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-26 · 3 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-27 · 3 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -8538,6 +8538,76 @@
           <t>🆕 NYTT
 2026-03-25
 🏛️ Platsbanken #30798017</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="55" customHeight="1">
+      <c r="A118" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B118" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C118" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D118" s="152" t="inlineStr">
+        <is>
+          <t>Östhammar</t>
+        </is>
+      </c>
+      <c r="E118" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F118" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G118" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H118" s="153" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I118" s="153" t="inlineStr">
+        <is>
+          <t>~49 km</t>
+        </is>
+      </c>
+      <c r="J118" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K118" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L118" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M118" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-26
+🏛️ Platsbanken #30802826</t>
         </is>
       </c>
     </row>
@@ -8629,6 +8699,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B116" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B117" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B118" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-03-31
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M125"/>
+  <dimension ref="A1:M126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-29 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-31 · 8 källor · Radie &lt;50 km · 1 nya · 3 borttagna</t>
         </is>
       </c>
     </row>
@@ -9070,6 +9070,76 @@
           <t>🆕 NYTT
 2026-12-11
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="55" customHeight="1">
+      <c r="A126" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B126" s="129" t="inlineStr">
+        <is>
+          <t>Nattassistent sökes till 14-årig pojke i Uppsala</t>
+        </is>
+      </c>
+      <c r="C126" s="152" t="inlineStr">
+        <is>
+          <t>Olivia Personlig Assistans AB</t>
+        </is>
+      </c>
+      <c r="D126" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E126" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F126" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G126" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H126" s="153" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="I126" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J126" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K126" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L126" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M126" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🏛️ Platsbanken #30819171</t>
         </is>
       </c>
     </row>
@@ -9169,6 +9239,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B123" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B124" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B125" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B126" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-04-01
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M126"/>
+  <dimension ref="A1:M128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-03-31 · 8 källor · Radie &lt;50 km · 1 nya · 3 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-01 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -9140,6 +9140,138 @@
           <t>🆕 NYTT
 2026-03-30
 🏛️ Platsbanken #30819171</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="55" customHeight="1">
+      <c r="A127" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B127" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C127" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D127" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E127" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F127" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G127" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H127" s="146" t="inlineStr"/>
+      <c r="I127" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J127" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K127" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L127" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M127" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="55" customHeight="1">
+      <c r="A128" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B128" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C128" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D128" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E128" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F128" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G128" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H128" s="146" t="inlineStr"/>
+      <c r="I128" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J128" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K128" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L128" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M128" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -9240,6 +9372,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B124" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B125" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B126" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B127" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B128" r:id="rId88"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-04-07
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M128"/>
+  <dimension ref="A1:M129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-01 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-07 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -9272,6 +9272,67 @@
           <t>🆕 NYTT
 2026-02-18
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="55" customHeight="1">
+      <c r="A129" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B129" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en ung pojke med NPF diagnoser i Uppsala</t>
+        </is>
+      </c>
+      <c r="C129" s="152" t="inlineStr"/>
+      <c r="D129" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E129" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F129" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G129" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H129" s="153" t="inlineStr"/>
+      <c r="I129" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J129" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K129" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L129" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M129" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -9374,6 +9435,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B126" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B127" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B128" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B129" r:id="rId89"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-04-11
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M129"/>
+  <dimension ref="A1:M130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-07 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-11 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -9333,6 +9333,76 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="55" customHeight="1">
+      <c r="A130" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B130" s="129" t="inlineStr">
+        <is>
+          <t>Trygg och lyhörd assistent sökes till man i Uppsala – timanställning</t>
+        </is>
+      </c>
+      <c r="C130" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D130" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E130" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F130" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G130" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H130" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I130" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J130" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K130" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L130" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M130" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-10
+🏛️ Platsbanken #30888235</t>
         </is>
       </c>
     </row>
@@ -9436,6 +9506,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B127" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B128" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B129" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B130" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-04-15
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M130"/>
+  <dimension ref="A1:M138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-14 · 8 källor · Radie &lt;50 km · 0 nya · 6 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-15 · 8 källor · Radie &lt;50 km · 8 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -9403,6 +9403,542 @@
           <t>🆕 NYTT
 2026-04-10
 🏛️ Platsbanken #30888235</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="55" customHeight="1">
+      <c r="A131" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B131" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C131" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D131" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E131" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F131" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G131" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H131" s="146" t="inlineStr"/>
+      <c r="I131" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J131" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K131" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L131" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M131" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="55" customHeight="1">
+      <c r="A132" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B132" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C132" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D132" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E132" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F132" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G132" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H132" s="146" t="inlineStr"/>
+      <c r="I132" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J132" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K132" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L132" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M132" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="55" customHeight="1">
+      <c r="A133" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B133" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C133" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D133" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E133" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F133" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G133" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H133" s="146" t="inlineStr"/>
+      <c r="I133" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J133" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K133" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L133" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M133" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="55" customHeight="1">
+      <c r="A134" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B134" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C134" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D134" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E134" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F134" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G134" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H134" s="146" t="inlineStr"/>
+      <c r="I134" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J134" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K134" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L134" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M134" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="55" customHeight="1">
+      <c r="A135" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B135" s="123" t="inlineStr">
+        <is>
+          <t>Extrajobb som personlig assistent till härlig kille i Knivsta</t>
+        </is>
+      </c>
+      <c r="C135" s="145" t="inlineStr">
+        <is>
+          <t>Vivida Assistans AB</t>
+        </is>
+      </c>
+      <c r="D135" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E135" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F135" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G135" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H135" s="146" t="inlineStr"/>
+      <c r="I135" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J135" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K135" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L135" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M135" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-01-07
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="55" customHeight="1">
+      <c r="A136" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B136" s="129" t="inlineStr">
+        <is>
+          <t>Assistent sökes till aktiv kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C136" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D136" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E136" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F136" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G136" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H136" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="I136" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J136" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K136" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L136" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M136" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-14
+🏛️ Platsbanken #30903817</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="55" customHeight="1">
+      <c r="A137" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B137" s="129" t="inlineStr">
+        <is>
+          <t>Humana söker personlig assistent till 23 årig kille i Uppsala!</t>
+        </is>
+      </c>
+      <c r="C137" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D137" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E137" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F137" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G137" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H137" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="I137" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J137" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K137" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L137" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M137" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-14
+🏛️ Platsbanken #30903402</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="55" customHeight="1">
+      <c r="A138" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B138" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C138" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D138" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E138" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F138" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G138" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H138" s="153" t="inlineStr"/>
+      <c r="I138" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J138" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K138" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L138" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M138" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -9507,6 +10043,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B128" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B129" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B130" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B131" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B132" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B133" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B134" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B135" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B136" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B137" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B138" r:id="rId98"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-04-18
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M138"/>
+  <dimension ref="A1:M139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-15 · 8 källor · Radie &lt;50 km · 8 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-18 · 8 källor · Radie &lt;50 km · 1 nya · 2 borttagna</t>
         </is>
       </c>
     </row>
@@ -9939,6 +9939,76 @@
           <t>🆕 NYTT
 2026-02-19
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="55" customHeight="1">
+      <c r="A139" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B139" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till en ung man i Uppsala inför sommaren 2026</t>
+        </is>
+      </c>
+      <c r="C139" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D139" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E139" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F139" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G139" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H139" s="153" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="I139" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J139" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K139" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L139" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M139" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🏛️ Platsbanken #30922617</t>
         </is>
       </c>
     </row>
@@ -10051,6 +10121,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B136" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B137" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B138" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B139" r:id="rId99"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-04-20
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M139"/>
+  <dimension ref="A1:M140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-19 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-20 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -10009,6 +10009,72 @@
           <t>🆕 NYTT
 2026-04-17
 🏛️ Platsbanken #30922617</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="55" customHeight="1">
+      <c r="A140" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B140" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C140" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D140" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E140" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F140" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G140" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H140" s="146" t="inlineStr"/>
+      <c r="I140" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J140" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K140" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L140" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M140" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -10122,6 +10188,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B137" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B138" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B139" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B140" r:id="rId100"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-04-22
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M140"/>
+  <dimension ref="A1:M142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-20 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-22 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -10075,6 +10075,146 @@
           <t>🆕 NYTT
 2026-02-23
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="55" customHeight="1">
+      <c r="A141" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B141" s="129" t="inlineStr">
+        <is>
+          <t>Assistent sökes till 3-årig pojke i Uppsala</t>
+        </is>
+      </c>
+      <c r="C141" s="152" t="inlineStr">
+        <is>
+          <t>Aberia AB</t>
+        </is>
+      </c>
+      <c r="D141" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E141" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F141" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G141" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H141" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="I141" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J141" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K141" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L141" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M141" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-21
+🏛️ Platsbanken #30932984</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="55" customHeight="1">
+      <c r="A142" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B142" s="133" t="inlineStr">
+        <is>
+          <t>Trygg och lyhörd assistent sökes till man i Tierp (timanställning)</t>
+        </is>
+      </c>
+      <c r="C142" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D142" s="157" t="inlineStr">
+        <is>
+          <t>timanställning) varaktighet: Behovsanställning Humana (Tierp</t>
+        </is>
+      </c>
+      <c r="E142" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F142" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G142" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H142" s="158" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="I142" s="158" t="inlineStr">
+        <is>
+          <t>~43 km</t>
+        </is>
+      </c>
+      <c r="J142" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K142" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L142" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M142" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-21
+🏛️ Platsbanken #30932351</t>
         </is>
       </c>
     </row>
@@ -10189,6 +10329,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B138" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B139" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B140" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B141" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B142" r:id="rId102"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-04-23
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M142"/>
+  <dimension ref="A1:M145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-22 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-23 · 8 källor · Radie &lt;50 km · 3 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -10215,6 +10215,212 @@
           <t>🆕 NYTT
 2026-04-21
 🏛️ Platsbanken #30932351</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="55" customHeight="1">
+      <c r="A143" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B143" s="129" t="inlineStr">
+        <is>
+          <t>Assistent med körkort sökes till kille</t>
+        </is>
+      </c>
+      <c r="C143" s="152" t="inlineStr">
+        <is>
+          <t>Nordin Assistans AB</t>
+        </is>
+      </c>
+      <c r="D143" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E143" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F143" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G143" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H143" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="I143" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J143" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K143" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L143" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M143" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-22
+🏛️ Platsbanken #30943916</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="55" customHeight="1">
+      <c r="A144" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B144" s="129" t="inlineStr">
+        <is>
+          <t>Assistent till Glad och Aktiv kille i Uppsala</t>
+        </is>
+      </c>
+      <c r="C144" s="152" t="inlineStr">
+        <is>
+          <t>Vår Omtanke Sverige AB</t>
+        </is>
+      </c>
+      <c r="D144" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E144" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F144" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G144" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H144" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I144" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J144" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K144" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L144" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M144" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-22
+🏛️ Platsbanken #30940418</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="55" customHeight="1">
+      <c r="A145" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B145" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C145" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D145" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E145" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F145" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G145" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H145" s="153" t="inlineStr"/>
+      <c r="I145" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J145" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K145" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L145" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M145" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -10331,6 +10537,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B140" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B141" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B142" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B143" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B144" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B145" r:id="rId105"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-05-01
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M145"/>
+  <dimension ref="A1:M147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-04-23 · 8 källor · Radie &lt;50 km · 3 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-01 · 8 källor · Radie &lt;50 km · 2 nya · 2 borttagna</t>
         </is>
       </c>
     </row>
@@ -10420,6 +10420,138 @@
         <is>
           <t>🆕 NYTT
 2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="55" customHeight="1">
+      <c r="A146" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B146" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C146" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D146" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E146" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F146" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G146" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H146" s="153" t="inlineStr"/>
+      <c r="I146" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J146" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K146" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L146" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M146" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="55" customHeight="1">
+      <c r="A147" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B147" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C147" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D147" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E147" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F147" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G147" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H147" s="153" t="inlineStr"/>
+      <c r="I147" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J147" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K147" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L147" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M147" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
 🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
@@ -10540,6 +10672,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B143" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B144" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B145" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B146" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B147" r:id="rId107"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-05-04
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M147"/>
+  <dimension ref="A1:M148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-01 · 8 källor · Radie &lt;50 km · 2 nya · 2 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-04 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -10552,6 +10552,72 @@
         <is>
           <t>🆕 NYTT
 2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="55" customHeight="1">
+      <c r="A148" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B148" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent- Uppsala</t>
+        </is>
+      </c>
+      <c r="C148" s="152" t="inlineStr">
+        <is>
+          <t>Inova Assistans AB</t>
+        </is>
+      </c>
+      <c r="D148" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E148" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F148" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G148" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H148" s="153" t="inlineStr"/>
+      <c r="I148" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J148" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K148" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L148" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M148" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-31
 🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
@@ -10674,6 +10740,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B145" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B146" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B147" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B148" r:id="rId108"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-05-07
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M148"/>
+  <dimension ref="A1:M149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-06 · 8 källor · Radie &lt;50 km · 0 nya · 2 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-07 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -10619,6 +10619,76 @@
           <t>🆕 NYTT
 2026-03-31
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="55" customHeight="1">
+      <c r="A149" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B149" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent till kille mellan Östervåla och Månkarbo</t>
+        </is>
+      </c>
+      <c r="C149" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D149" s="157" t="inlineStr">
+        <is>
+          <t>Heby</t>
+        </is>
+      </c>
+      <c r="E149" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F149" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G149" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H149" s="158" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="I149" s="158" t="inlineStr">
+        <is>
+          <t>~47 km</t>
+        </is>
+      </c>
+      <c r="J149" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K149" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L149" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M149" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-05-06
+🏛️ Platsbanken #31003754</t>
         </is>
       </c>
     </row>
@@ -10741,6 +10811,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B146" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B147" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B148" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B149" r:id="rId109"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-05-13
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M149"/>
+  <dimension ref="A1:M150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-12 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-13 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -10689,6 +10689,76 @@
           <t>🆕 NYTT
 2026-05-06
 🏛️ Platsbanken #31003754</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="55" customHeight="1">
+      <c r="A150" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B150" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie och engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C150" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D150" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E150" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F150" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G150" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H150" s="153" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="I150" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J150" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K150" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L150" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M150" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-05-12
+🏛️ Platsbanken #31026562</t>
         </is>
       </c>
     </row>
@@ -10812,6 +10882,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B147" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B148" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B149" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B150" r:id="rId110"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-05-16
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M150"/>
+  <dimension ref="A1:M161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-14 · 8 källor · Radie &lt;50 km · 0 nya · 12 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-16 · 8 källor · Radie &lt;50 km · 11 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -10759,6 +10759,776 @@
           <t>🆕 NYTT
 2026-05-12
 🏛️ Platsbanken #31026562</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="55" customHeight="1">
+      <c r="A151" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B151" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C151" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D151" s="145" t="inlineStr">
+        <is>
+          <t>Tierp</t>
+        </is>
+      </c>
+      <c r="E151" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F151" s="145" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G151" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H151" s="146" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I151" s="146" t="inlineStr">
+        <is>
+          <t>~43 km</t>
+        </is>
+      </c>
+      <c r="J151" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K151" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L151" s="150" t="inlineStr">
+        <is>
+          <t>🟠
+Sök INNAN semestern.</t>
+        </is>
+      </c>
+      <c r="M151" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-26
+🏛️ Platsbanken #30666709</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="55" customHeight="1">
+      <c r="A152" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B152" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie och engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C152" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D152" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E152" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F152" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G152" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H152" s="153" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="I152" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J152" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K152" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L152" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M152" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-05-12
+🏛️ Platsbanken #31026562</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="55" customHeight="1">
+      <c r="A153" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B153" s="129" t="inlineStr">
+        <is>
+          <t>Assistent med körkort sökes till kille</t>
+        </is>
+      </c>
+      <c r="C153" s="152" t="inlineStr">
+        <is>
+          <t>Nordin Assistans AB</t>
+        </is>
+      </c>
+      <c r="D153" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E153" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F153" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G153" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H153" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="I153" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J153" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K153" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L153" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M153" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-22
+🏛️ Platsbanken #30943916</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="55" customHeight="1">
+      <c r="A154" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B154" s="129" t="inlineStr">
+        <is>
+          <t>Assistent till Glad och Aktiv kille i Uppsala</t>
+        </is>
+      </c>
+      <c r="C154" s="152" t="inlineStr">
+        <is>
+          <t>Vår Omtanke Sverige AB</t>
+        </is>
+      </c>
+      <c r="D154" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E154" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F154" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G154" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H154" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I154" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J154" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K154" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L154" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M154" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-22
+🏛️ Platsbanken #30940418</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="55" customHeight="1">
+      <c r="A155" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B155" s="129" t="inlineStr">
+        <is>
+          <t>Assistent sökes till 3-årig pojke i Uppsala</t>
+        </is>
+      </c>
+      <c r="C155" s="152" t="inlineStr">
+        <is>
+          <t>Aberia AB</t>
+        </is>
+      </c>
+      <c r="D155" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E155" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F155" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G155" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H155" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="I155" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J155" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K155" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L155" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M155" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-21
+🏛️ Platsbanken #30932984</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="55" customHeight="1">
+      <c r="A156" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B156" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till en ung man i Uppsala inför sommaren 2026</t>
+        </is>
+      </c>
+      <c r="C156" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D156" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E156" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F156" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G156" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H156" s="153" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="I156" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J156" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K156" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L156" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M156" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🏛️ Platsbanken #30922617</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="55" customHeight="1">
+      <c r="A157" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B157" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C157" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D157" s="152" t="inlineStr">
+        <is>
+          <t>Östhammar</t>
+        </is>
+      </c>
+      <c r="E157" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F157" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G157" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H157" s="153" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I157" s="153" t="inlineStr">
+        <is>
+          <t>~49 km</t>
+        </is>
+      </c>
+      <c r="J157" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K157" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L157" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M157" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-26
+🏛️ Platsbanken #30802826</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="55" customHeight="1">
+      <c r="A158" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B158" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till aktiv man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C158" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D158" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E158" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F158" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G158" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H158" s="153" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="I158" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J158" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K158" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L158" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M158" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-24
+🏛️ Platsbanken #30791374</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="55" customHeight="1">
+      <c r="A159" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B159" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C159" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D159" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E159" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F159" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G159" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H159" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I159" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J159" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K159" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L159" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M159" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-19
+🏛️ Platsbanken #30769628</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="55" customHeight="1">
+      <c r="A160" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B160" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C160" s="152" t="inlineStr">
+        <is>
+          <t>Inkludera Assistans AB</t>
+        </is>
+      </c>
+      <c r="D160" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E160" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F160" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G160" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H160" s="153" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="I160" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J160" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K160" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L160" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M160" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-03
+🏛️ Platsbanken #30687806</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="55" customHeight="1">
+      <c r="A161" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B161" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent till kille mellan Östervåla och Månkarbo</t>
+        </is>
+      </c>
+      <c r="C161" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D161" s="157" t="inlineStr">
+        <is>
+          <t>Heby</t>
+        </is>
+      </c>
+      <c r="E161" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F161" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G161" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H161" s="158" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="I161" s="158" t="inlineStr">
+        <is>
+          <t>~47 km</t>
+        </is>
+      </c>
+      <c r="J161" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K161" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L161" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M161" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-05-06
+🏛️ Platsbanken #31003754</t>
         </is>
       </c>
     </row>
@@ -10883,6 +11653,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B148" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B149" r:id="rId109"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B150" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B151" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B152" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B153" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B154" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B155" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B156" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B157" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B158" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B159" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B160" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B161" r:id="rId121"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-05-19
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M161"/>
+  <dimension ref="A1:M162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-16 · 8 källor · Radie &lt;50 km · 11 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-19 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -11529,6 +11529,76 @@
           <t>🆕 NYTT
 2026-05-06
 🏛️ Platsbanken #31003754</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="55" customHeight="1">
+      <c r="A162" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B162" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till autistisk man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C162" s="152" t="inlineStr">
+        <is>
+          <t>Vår Omtanke Sverige AB</t>
+        </is>
+      </c>
+      <c r="D162" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E162" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F162" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G162" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H162" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="I162" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J162" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K162" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L162" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Diskutera semester.</t>
+        </is>
+      </c>
+      <c r="M162" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-05-18
+🏛️ Platsbanken #31045503</t>
         </is>
       </c>
     </row>
@@ -11664,6 +11734,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B159" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B160" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B161" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B162" r:id="rId122"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-05-21
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M162"/>
+  <dimension ref="A1:M165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-19 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-21 · 8 källor · Radie &lt;50 km · 3 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -11599,6 +11599,189 @@
           <t>🆕 NYTT
 2026-05-18
 🏛️ Platsbanken #31045503</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="55" customHeight="1">
+      <c r="A163" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B163" s="129" t="inlineStr">
+        <is>
+          <t>Assistenter sökes till en trevlig man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C163" s="152" t="inlineStr"/>
+      <c r="D163" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E163" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F163" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G163" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H163" s="153" t="inlineStr"/>
+      <c r="I163" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J163" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K163" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L163" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M163" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="55" customHeight="1">
+      <c r="A164" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B164" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till en ung man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C164" s="152" t="inlineStr"/>
+      <c r="D164" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E164" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F164" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G164" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H164" s="153" t="inlineStr"/>
+      <c r="I164" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J164" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K164" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L164" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M164" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="55" customHeight="1">
+      <c r="A165" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B165" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till vuxen man</t>
+        </is>
+      </c>
+      <c r="C165" s="152" t="inlineStr"/>
+      <c r="D165" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E165" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F165" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G165" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H165" s="153" t="inlineStr"/>
+      <c r="I165" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J165" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K165" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L165" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M165" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -11735,6 +11918,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B160" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B161" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B162" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B163" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B164" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B165" r:id="rId125"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-05-26
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M165"/>
+  <dimension ref="A1:M167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-23 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-26 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -11782,6 +11782,146 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="55" customHeight="1">
+      <c r="A166" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B166" s="129" t="inlineStr">
+        <is>
+          <t>Assistenter sökes till en trevlig man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C166" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D166" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E166" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F166" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G166" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H166" s="153" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I166" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J166" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K166" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L166" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M166" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-05-20
+🏛️ Platsbanken #31062823</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="55" customHeight="1">
+      <c r="A167" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B167" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent åt kille i Östervåla</t>
+        </is>
+      </c>
+      <c r="C167" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D167" s="157" t="inlineStr">
+        <is>
+          <t>Tierp</t>
+        </is>
+      </c>
+      <c r="E167" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F167" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G167" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H167" s="158" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="I167" s="158" t="inlineStr">
+        <is>
+          <t>~43 km</t>
+        </is>
+      </c>
+      <c r="J167" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K167" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L167" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M167" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-05-25
+🏛️ Platsbanken #31077869</t>
         </is>
       </c>
     </row>
@@ -11921,6 +12061,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B163" r:id="rId123"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B164" r:id="rId124"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B165" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B166" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B167" r:id="rId127"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-05-30
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M167"/>
+  <dimension ref="A1:M169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-28 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-30 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -11922,6 +11922,146 @@
           <t>🆕 NYTT
 2026-05-25
 🏛️ Platsbanken #31077869</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="55" customHeight="1">
+      <c r="A168" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B168" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till en 20-årig kille med autism och IF.</t>
+        </is>
+      </c>
+      <c r="C168" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D168" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E168" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F168" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G168" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H168" s="153" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="I168" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J168" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K168" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L168" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M168" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-05-29
+🏛️ Platsbanken #31101996</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="55" customHeight="1">
+      <c r="A169" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B169" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent, timvikariat, sökes till man i Heby</t>
+        </is>
+      </c>
+      <c r="C169" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D169" s="157" t="inlineStr">
+        <is>
+          <t>Heby</t>
+        </is>
+      </c>
+      <c r="E169" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F169" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G169" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H169" s="158" t="inlineStr">
+        <is>
+          <t>2026-11-25</t>
+        </is>
+      </c>
+      <c r="I169" s="158" t="inlineStr">
+        <is>
+          <t>~47 km</t>
+        </is>
+      </c>
+      <c r="J169" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K169" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L169" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M169" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-05-29
+🏛️ Platsbanken #31105052</t>
         </is>
       </c>
     </row>
@@ -12063,6 +12203,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B165" r:id="rId125"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B166" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B167" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B168" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B169" r:id="rId129"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-01
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M169"/>
+  <dimension ref="A1:M174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-05-30 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-01 · 8 källor · Radie &lt;50 km · 5 nya · 4 borttagna</t>
         </is>
       </c>
     </row>
@@ -12062,6 +12062,340 @@
           <t>🆕 NYTT
 2026-05-29
 🏛️ Platsbanken #31105052</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="55" customHeight="1">
+      <c r="A170" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B170" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C170" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D170" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E170" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F170" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G170" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H170" s="146" t="inlineStr"/>
+      <c r="I170" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J170" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K170" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L170" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M170" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="55" customHeight="1">
+      <c r="A171" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B171" s="123" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C171" s="145" t="inlineStr">
+        <is>
+          <t>Inkludera assistans i Sverige AB</t>
+        </is>
+      </c>
+      <c r="D171" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E171" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F171" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G171" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H171" s="146" t="inlineStr"/>
+      <c r="I171" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J171" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K171" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L171" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M171" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-03
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="55" customHeight="1">
+      <c r="A172" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B172" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till en ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C172" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D172" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E172" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F172" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G172" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H172" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-28</t>
+        </is>
+      </c>
+      <c r="I172" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J172" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K172" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L172" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M172" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-01
+🏛️ Platsbanken #31111080</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="55" customHeight="1">
+      <c r="A173" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B173" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C173" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D173" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E173" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F173" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G173" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H173" s="153" t="inlineStr"/>
+      <c r="I173" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J173" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K173" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L173" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M173" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="55" customHeight="1">
+      <c r="A174" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B174" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C174" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D174" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E174" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F174" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G174" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H174" s="153" t="inlineStr"/>
+      <c r="I174" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J174" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K174" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L174" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M174" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -12205,6 +12539,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B167" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B168" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B169" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B170" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B171" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B172" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B173" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B174" r:id="rId134"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-03
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M174"/>
+  <dimension ref="A1:M189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-02 · 8 källor · Radie &lt;50 km · 0 nya · 14 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-03 · 8 källor · Radie &lt;50 km · 15 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -12395,6 +12395,995 @@
         <is>
           <t>🆕 NYTT
 2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="55" customHeight="1">
+      <c r="A175" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B175" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C175" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D175" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E175" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F175" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G175" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H175" s="146" t="inlineStr"/>
+      <c r="I175" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J175" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K175" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L175" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M175" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="55" customHeight="1">
+      <c r="A176" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B176" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C176" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D176" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E176" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F176" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G176" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H176" s="146" t="inlineStr"/>
+      <c r="I176" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J176" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K176" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L176" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M176" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="55" customHeight="1">
+      <c r="A177" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B177" s="123" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C177" s="145" t="inlineStr">
+        <is>
+          <t>Inkludera assistans i Sverige AB</t>
+        </is>
+      </c>
+      <c r="D177" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E177" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F177" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G177" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H177" s="146" t="inlineStr"/>
+      <c r="I177" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J177" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K177" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L177" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M177" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-03
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="55" customHeight="1">
+      <c r="A178" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B178" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C178" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D178" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E178" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F178" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G178" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H178" s="146" t="inlineStr"/>
+      <c r="I178" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J178" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K178" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L178" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M178" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="55" customHeight="1">
+      <c r="A179" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B179" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C179" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D179" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E179" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F179" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G179" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H179" s="146" t="inlineStr"/>
+      <c r="I179" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J179" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K179" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L179" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M179" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="55" customHeight="1">
+      <c r="A180" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B180" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C180" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D180" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E180" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F180" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G180" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H180" s="146" t="inlineStr"/>
+      <c r="I180" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J180" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K180" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L180" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M180" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="55" customHeight="1">
+      <c r="A181" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B181" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C181" s="152" t="inlineStr">
+        <is>
+          <t>Vivant Assistans AB</t>
+        </is>
+      </c>
+      <c r="D181" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E181" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F181" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G181" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H181" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-29</t>
+        </is>
+      </c>
+      <c r="I181" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J181" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K181" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L181" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M181" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-02
+🏛️ Platsbanken #31129740</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="55" customHeight="1">
+      <c r="A182" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B182" s="129" t="inlineStr">
+        <is>
+          <t>Social man i 70-års åldern söker personlig assistent</t>
+        </is>
+      </c>
+      <c r="C182" s="152" t="inlineStr"/>
+      <c r="D182" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E182" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F182" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G182" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H182" s="153" t="inlineStr"/>
+      <c r="I182" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J182" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K182" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L182" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M182" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="55" customHeight="1">
+      <c r="A183" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B183" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C183" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D183" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E183" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F183" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G183" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H183" s="153" t="inlineStr"/>
+      <c r="I183" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J183" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K183" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L183" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M183" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="55" customHeight="1">
+      <c r="A184" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B184" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C184" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D184" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E184" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F184" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G184" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H184" s="153" t="inlineStr"/>
+      <c r="I184" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J184" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K184" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L184" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M184" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="55" customHeight="1">
+      <c r="A185" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B185" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C185" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D185" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E185" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F185" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G185" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H185" s="153" t="inlineStr"/>
+      <c r="I185" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J185" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K185" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L185" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M185" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="55" customHeight="1">
+      <c r="A186" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B186" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C186" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D186" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E186" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F186" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G186" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H186" s="153" t="inlineStr"/>
+      <c r="I186" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J186" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K186" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L186" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M186" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="55" customHeight="1">
+      <c r="A187" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B187" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C187" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D187" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E187" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F187" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G187" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H187" s="153" t="inlineStr"/>
+      <c r="I187" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J187" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K187" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L187" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M187" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="55" customHeight="1">
+      <c r="A188" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B188" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C188" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D188" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E188" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F188" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G188" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H188" s="153" t="inlineStr"/>
+      <c r="I188" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J188" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K188" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L188" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M188" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="55" customHeight="1">
+      <c r="A189" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B189" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C189" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D189" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E189" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F189" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G189" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H189" s="153" t="inlineStr"/>
+      <c r="I189" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J189" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K189" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L189" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M189" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
 🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
@@ -12544,6 +13533,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B172" r:id="rId132"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B173" r:id="rId133"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B174" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B175" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B176" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B177" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B178" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B179" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B180" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B181" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B182" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B183" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B184" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B185" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B186" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B187" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B188" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B189" r:id="rId149"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-04
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M189"/>
+  <dimension ref="A1:M192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-03 · 8 källor · Radie &lt;50 km · 15 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-04 · 8 källor · Radie &lt;50 km · 3 nya · 2 borttagna</t>
         </is>
       </c>
     </row>
@@ -13385,6 +13385,198 @@
           <t>🆕 NYTT
 2026-02-19
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="55" customHeight="1">
+      <c r="A190" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B190" s="129" t="inlineStr">
+        <is>
+          <t>Social man i 70-års åldern söker personlig assistent</t>
+        </is>
+      </c>
+      <c r="C190" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D190" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E190" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F190" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G190" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H190" s="153" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="I190" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J190" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K190" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L190" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M190" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-03
+🏛️ Platsbanken #31131605</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="55" customHeight="1">
+      <c r="A191" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B191" s="129" t="inlineStr">
+        <is>
+          <t>Assistent sökes till 3-årig pojke i Uppsala</t>
+        </is>
+      </c>
+      <c r="C191" s="152" t="inlineStr"/>
+      <c r="D191" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E191" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F191" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G191" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H191" s="153" t="inlineStr"/>
+      <c r="I191" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J191" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K191" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L191" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M191" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="55" customHeight="1">
+      <c r="A192" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B192" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till aktiv man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C192" s="152" t="inlineStr"/>
+      <c r="D192" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E192" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F192" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G192" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H192" s="153" t="inlineStr"/>
+      <c r="I192" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J192" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K192" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L192" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M192" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -13548,6 +13740,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B187" r:id="rId147"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B188" r:id="rId148"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B189" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B190" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B191" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B192" r:id="rId152"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-05
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M192"/>
+  <dimension ref="A1:M197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-04 · 8 källor · Radie &lt;50 km · 3 nya · 2 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-05 · 8 källor · Radie &lt;50 km · 5 nya · 3 borttagna</t>
         </is>
       </c>
     </row>
@@ -13577,6 +13577,356 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="55" customHeight="1">
+      <c r="A193" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B193" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C193" s="152" t="inlineStr">
+        <is>
+          <t>Inkludera Assistans AB</t>
+        </is>
+      </c>
+      <c r="D193" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E193" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F193" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G193" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H193" s="153" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="I193" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J193" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K193" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L193" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M193" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-04
+🏛️ Platsbanken #31141991</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="55" customHeight="1">
+      <c r="A194" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B194" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till man i Uppsala - två tjänster</t>
+        </is>
+      </c>
+      <c r="C194" s="152" t="inlineStr">
+        <is>
+          <t>Livsam Personlig Assistans AB</t>
+        </is>
+      </c>
+      <c r="D194" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E194" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F194" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G194" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H194" s="153" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I194" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J194" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K194" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L194" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M194" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-04
+🏛️ Platsbanken #31139830</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="55" customHeight="1">
+      <c r="A195" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B195" s="129" t="inlineStr">
+        <is>
+          <t>Assistent sökes till 3-årig pojke i Uppsala</t>
+        </is>
+      </c>
+      <c r="C195" s="152" t="inlineStr">
+        <is>
+          <t>Aberia AB</t>
+        </is>
+      </c>
+      <c r="D195" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E195" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F195" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G195" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H195" s="153" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="I195" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J195" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K195" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L195" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M195" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-04
+🏛️ Platsbanken #31138562</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="55" customHeight="1">
+      <c r="A196" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B196" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till aktiv man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C196" s="152" t="inlineStr">
+        <is>
+          <t>Vivant Assistans AB</t>
+        </is>
+      </c>
+      <c r="D196" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E196" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F196" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G196" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H196" s="153" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I196" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J196" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K196" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L196" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M196" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-04
+🏛️ Platsbanken #31138342</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="55" customHeight="1">
+      <c r="A197" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B197" s="133" t="inlineStr">
+        <is>
+          <t>Trygg och lyhörd assistent sökes till man i Tierp (timanställning)</t>
+        </is>
+      </c>
+      <c r="C197" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D197" s="157" t="inlineStr">
+        <is>
+          <t>timanställning) varaktighet: Behovsanställning Humana (Tierp</t>
+        </is>
+      </c>
+      <c r="E197" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F197" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G197" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H197" s="158" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="I197" s="158" t="inlineStr">
+        <is>
+          <t>~43 km</t>
+        </is>
+      </c>
+      <c r="J197" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K197" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L197" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M197" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-04
+🏛️ Platsbanken #31138478</t>
         </is>
       </c>
     </row>
@@ -13743,6 +14093,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B190" r:id="rId150"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B191" r:id="rId151"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B192" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B193" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B194" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B195" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B196" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B197" r:id="rId157"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-08
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M197"/>
+  <dimension ref="A1:M198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-05 · 8 källor · Radie &lt;50 km · 5 nya · 3 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-08 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -13927,6 +13927,67 @@
           <t>🆕 NYTT
 2026-06-04
 🏛️ Platsbanken #31138478</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="55" customHeight="1">
+      <c r="A198" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B198" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till en ung man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C198" s="152" t="inlineStr"/>
+      <c r="D198" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E198" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F198" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G198" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H198" s="153" t="inlineStr"/>
+      <c r="I198" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J198" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K198" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L198" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M198" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -14098,6 +14159,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B195" r:id="rId155"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B196" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B197" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B198" r:id="rId158"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-09
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M198"/>
+  <dimension ref="A1:M199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-08 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-09 · 8 källor · Radie &lt;50 km · 1 nya · 2 borttagna</t>
         </is>
       </c>
     </row>
@@ -13988,6 +13988,76 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="55" customHeight="1">
+      <c r="A199" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B199" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvikarie sökes till 32-årig mjukvaruutvecklare i Uppsala</t>
+        </is>
+      </c>
+      <c r="C199" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D199" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E199" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F199" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G199" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H199" s="153" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="I199" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J199" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K199" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L199" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M199" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-08
+🏛️ Platsbanken #31150980</t>
         </is>
       </c>
     </row>
@@ -14160,6 +14230,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B196" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B197" r:id="rId157"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B198" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B199" r:id="rId159"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-15
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M199"/>
+  <dimension ref="A1:M200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-13 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-15 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -14058,6 +14058,67 @@
           <t>🆕 NYTT
 2026-06-08
 🏛️ Platsbanken #31150980</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="55" customHeight="1">
+      <c r="A200" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B200" s="129" t="inlineStr">
+        <is>
+          <t>NyTimvikarie och engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C200" s="152" t="inlineStr"/>
+      <c r="D200" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E200" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F200" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G200" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H200" s="153" t="inlineStr"/>
+      <c r="I200" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J200" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K200" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L200" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M200" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -14231,6 +14292,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B197" r:id="rId157"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B198" r:id="rId158"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B199" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B200" r:id="rId160"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-17
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M200"/>
+  <dimension ref="A1:M201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-16 · 8 källor · Radie &lt;50 km · 0 nya · 13 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-17 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -14116,6 +14116,67 @@
         </is>
       </c>
       <c r="M200" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="55" customHeight="1">
+      <c r="A201" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B201" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till en ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C201" s="152" t="inlineStr"/>
+      <c r="D201" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E201" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F201" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G201" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H201" s="153" t="inlineStr"/>
+      <c r="I201" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J201" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K201" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L201" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M201" s="154" t="inlineStr">
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
@@ -14293,6 +14354,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B198" r:id="rId158"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B199" r:id="rId159"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B200" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B201" r:id="rId161"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-18
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M201"/>
+  <dimension ref="A1:M213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-17 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-18 · 8 källor · Radie &lt;50 km · 12 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -14180,6 +14180,802 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="55" customHeight="1">
+      <c r="A202" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B202" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C202" s="145" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D202" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E202" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F202" s="145" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G202" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H202" s="146" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I202" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J202" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · ❓</t>
+        </is>
+      </c>
+      <c r="K202" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L202" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M202" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-17
+🏛️ Platsbanken #31189334</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="55" customHeight="1">
+      <c r="A203" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B203" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C203" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D203" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E203" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F203" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G203" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H203" s="146" t="inlineStr"/>
+      <c r="I203" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J203" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K203" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L203" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M203" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="55" customHeight="1">
+      <c r="A204" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B204" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C204" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D204" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E204" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F204" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G204" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H204" s="146" t="inlineStr"/>
+      <c r="I204" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J204" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K204" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L204" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M204" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="55" customHeight="1">
+      <c r="A205" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B205" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C205" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D205" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E205" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F205" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G205" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H205" s="146" t="inlineStr"/>
+      <c r="I205" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J205" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K205" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L205" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M205" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="55" customHeight="1">
+      <c r="A206" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B206" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C206" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D206" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E206" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F206" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G206" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H206" s="146" t="inlineStr"/>
+      <c r="I206" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J206" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K206" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L206" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M206" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="55" customHeight="1">
+      <c r="A207" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B207" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C207" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D207" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E207" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F207" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G207" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H207" s="153" t="inlineStr"/>
+      <c r="I207" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J207" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K207" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L207" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M207" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="55" customHeight="1">
+      <c r="A208" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B208" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C208" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D208" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E208" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F208" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G208" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H208" s="153" t="inlineStr"/>
+      <c r="I208" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J208" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K208" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L208" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M208" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="55" customHeight="1">
+      <c r="A209" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B209" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C209" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D209" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E209" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F209" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G209" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H209" s="153" t="inlineStr"/>
+      <c r="I209" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J209" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K209" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L209" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M209" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="55" customHeight="1">
+      <c r="A210" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B210" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C210" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D210" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E210" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F210" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G210" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H210" s="153" t="inlineStr"/>
+      <c r="I210" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J210" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K210" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L210" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M210" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" ht="55" customHeight="1">
+      <c r="A211" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B211" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C211" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D211" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E211" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F211" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G211" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H211" s="153" t="inlineStr"/>
+      <c r="I211" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J211" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K211" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L211" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M211" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="55" customHeight="1">
+      <c r="A212" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B212" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C212" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D212" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E212" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F212" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G212" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H212" s="153" t="inlineStr"/>
+      <c r="I212" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J212" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K212" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L212" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M212" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="55" customHeight="1">
+      <c r="A213" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B213" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C213" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D213" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E213" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F213" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G213" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H213" s="153" t="inlineStr"/>
+      <c r="I213" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J213" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K213" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L213" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M213" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -14355,6 +15151,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B199" r:id="rId159"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B200" r:id="rId160"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B201" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B202" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B203" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B204" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B205" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B206" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B207" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B208" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B209" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B210" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B211" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B212" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B213" r:id="rId173"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-19
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M213"/>
+  <dimension ref="A1:M214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-18 · 8 källor · Radie &lt;50 km · 12 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-19 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -14976,6 +14976,76 @@
           <t>🆕 NYTT
 2026-02-19
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" ht="55" customHeight="1">
+      <c r="A214" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B214" s="133" t="inlineStr">
+        <is>
+          <t>Initiativrik assistent sökes till 8-årig kille</t>
+        </is>
+      </c>
+      <c r="C214" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D214" s="157" t="inlineStr">
+        <is>
+          <t>Östhammar</t>
+        </is>
+      </c>
+      <c r="E214" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F214" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G214" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H214" s="158" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I214" s="158" t="inlineStr">
+        <is>
+          <t>~49 km</t>
+        </is>
+      </c>
+      <c r="J214" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K214" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L214" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M214" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-18
+🏛️ Platsbanken #31193785</t>
         </is>
       </c>
     </row>
@@ -15163,6 +15233,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B211" r:id="rId171"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B212" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B213" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B214" r:id="rId174"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-23
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M214"/>
+  <dimension ref="A1:M218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-19 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-23 · 8 källor · Radie &lt;50 km · 4 nya · 2 borttagna</t>
         </is>
       </c>
     </row>
@@ -15046,6 +15046,268 @@
           <t>🆕 NYTT
 2026-06-18
 🏛️ Platsbanken #31193785</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" ht="55" customHeight="1">
+      <c r="A215" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B215" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till man i Uppsala - fast schemarad</t>
+        </is>
+      </c>
+      <c r="C215" s="152" t="inlineStr">
+        <is>
+          <t>Livsam Personlig Assistans AB</t>
+        </is>
+      </c>
+      <c r="D215" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E215" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F215" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G215" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H215" s="153" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I215" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J215" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K215" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L215" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M215" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-23
+🏛️ Platsbanken #31204799</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="55" customHeight="1">
+      <c r="A216" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B216" s="129" t="inlineStr">
+        <is>
+          <t>Man i Uppsala söker assistans 15:00-21:00 mån-fre.</t>
+        </is>
+      </c>
+      <c r="C216" s="152" t="inlineStr">
+        <is>
+          <t>God Assistans i Mitt AB</t>
+        </is>
+      </c>
+      <c r="D216" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E216" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F216" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G216" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H216" s="153" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I216" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J216" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K216" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L216" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Diskutera semester.</t>
+        </is>
+      </c>
+      <c r="M216" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-06-23
+🏛️ Platsbanken #31203770</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" ht="55" customHeight="1">
+      <c r="A217" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B217" s="129" t="inlineStr">
+        <is>
+          <t>NyPersonlig assistent sökes till man i Uppsala - fast schemarad</t>
+        </is>
+      </c>
+      <c r="C217" s="152" t="inlineStr"/>
+      <c r="D217" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E217" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F217" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G217" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H217" s="153" t="inlineStr"/>
+      <c r="I217" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J217" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K217" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L217" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M217" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="55" customHeight="1">
+      <c r="A218" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B218" s="129" t="inlineStr">
+        <is>
+          <t>NyMan i Uppsala söker assistans 15:00-21:00 mån-fre.</t>
+        </is>
+      </c>
+      <c r="C218" s="152" t="inlineStr"/>
+      <c r="D218" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E218" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F218" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G218" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H218" s="153" t="inlineStr"/>
+      <c r="I218" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J218" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K218" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L218" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M218" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -15234,6 +15496,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B212" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B213" r:id="rId173"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B214" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B215" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B216" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B217" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B218" r:id="rId178"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-28
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M218"/>
+  <dimension ref="A1:M230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-26 · 8 källor · Radie &lt;50 km · 0 nya · 13 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-28 · 8 källor · Radie &lt;50 km · 12 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -15308,6 +15308,798 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="55" customHeight="1">
+      <c r="A219" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B219" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C219" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D219" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E219" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F219" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G219" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H219" s="146" t="inlineStr"/>
+      <c r="I219" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J219" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K219" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L219" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M219" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" ht="55" customHeight="1">
+      <c r="A220" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B220" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C220" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D220" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E220" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F220" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G220" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H220" s="146" t="inlineStr"/>
+      <c r="I220" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J220" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K220" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L220" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M220" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" ht="55" customHeight="1">
+      <c r="A221" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B221" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C221" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D221" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E221" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F221" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G221" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H221" s="146" t="inlineStr"/>
+      <c r="I221" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J221" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K221" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L221" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M221" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" ht="55" customHeight="1">
+      <c r="A222" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B222" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C222" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D222" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E222" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F222" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G222" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H222" s="146" t="inlineStr"/>
+      <c r="I222" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J222" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K222" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L222" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M222" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="55" customHeight="1">
+      <c r="A223" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B223" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C223" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D223" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E223" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F223" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G223" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H223" s="153" t="inlineStr"/>
+      <c r="I223" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J223" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K223" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L223" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M223" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="55" customHeight="1">
+      <c r="A224" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B224" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C224" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D224" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E224" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F224" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G224" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H224" s="153" t="inlineStr"/>
+      <c r="I224" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J224" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K224" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L224" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M224" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="55" customHeight="1">
+      <c r="A225" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B225" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent- Uppsala</t>
+        </is>
+      </c>
+      <c r="C225" s="152" t="inlineStr">
+        <is>
+          <t>Inova Assistans AB</t>
+        </is>
+      </c>
+      <c r="D225" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E225" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F225" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G225" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H225" s="153" t="inlineStr"/>
+      <c r="I225" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J225" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K225" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L225" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M225" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-31
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="55" customHeight="1">
+      <c r="A226" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B226" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C226" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D226" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E226" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F226" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G226" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H226" s="153" t="inlineStr"/>
+      <c r="I226" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J226" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K226" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L226" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M226" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="55" customHeight="1">
+      <c r="A227" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B227" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C227" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D227" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E227" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F227" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G227" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H227" s="153" t="inlineStr"/>
+      <c r="I227" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J227" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K227" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L227" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M227" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="55" customHeight="1">
+      <c r="A228" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B228" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C228" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D228" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E228" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F228" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G228" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H228" s="153" t="inlineStr"/>
+      <c r="I228" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J228" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K228" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L228" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M228" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="55" customHeight="1">
+      <c r="A229" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B229" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C229" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D229" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E229" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F229" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G229" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H229" s="153" t="inlineStr"/>
+      <c r="I229" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J229" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K229" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L229" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M229" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="55" customHeight="1">
+      <c r="A230" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B230" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C230" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D230" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E230" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F230" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G230" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H230" s="153" t="inlineStr"/>
+      <c r="I230" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J230" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K230" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L230" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M230" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -15500,6 +16292,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B216" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B217" r:id="rId177"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B218" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B219" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B220" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B221" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B222" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B223" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B224" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B225" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B226" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B227" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B228" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B229" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B230" r:id="rId190"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-06-30
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M230"/>
+  <dimension ref="A1:M231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-29 · 8 källor · Radie &lt;50 km · 0 nya · 2 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-30 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -16100,6 +16100,76 @@
           <t>🆕 NYTT
 2026-02-19
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="55" customHeight="1">
+      <c r="A231" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B231" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till aktiv man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C231" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D231" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E231" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F231" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G231" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H231" s="153" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="I231" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J231" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K231" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L231" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M231" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-24
+🏛️ Platsbanken #30791374</t>
         </is>
       </c>
     </row>
@@ -16304,6 +16374,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B228" r:id="rId188"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B229" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B230" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B231" r:id="rId191"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-07-01
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M231"/>
+  <dimension ref="A1:M233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-06-30 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-01 · 8 källor · Radie &lt;50 km · 2 nya · 2 borttagna</t>
         </is>
       </c>
     </row>
@@ -16170,6 +16170,137 @@
           <t>🆕 NYTT
 2026-03-24
 🏛️ Platsbanken #30791374</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="55" customHeight="1">
+      <c r="A232" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B232" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C232" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D232" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E232" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F232" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G232" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H232" s="146" t="inlineStr"/>
+      <c r="I232" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J232" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K232" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L232" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M232" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="55" customHeight="1">
+      <c r="A233" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B233" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till aktiv man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C233" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D233" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E233" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F233" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G233" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H233" s="153" t="inlineStr"/>
+      <c r="I233" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J233" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K233" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L233" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M233" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -16375,6 +16506,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B229" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B230" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B231" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B232" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B233" r:id="rId193"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-07-03
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M233"/>
+  <dimension ref="A1:M247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-02 · 8 källor · Radie &lt;50 km · 0 nya · 14 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-03 · 8 källor · Radie &lt;50 km · 14 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -16300,6 +16300,929 @@
         <is>
           <t>🆕 NYTT
 2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="55" customHeight="1">
+      <c r="A234" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B234" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C234" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D234" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E234" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F234" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G234" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H234" s="146" t="inlineStr"/>
+      <c r="I234" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J234" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K234" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L234" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M234" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="55" customHeight="1">
+      <c r="A235" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B235" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C235" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D235" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E235" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F235" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G235" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H235" s="146" t="inlineStr"/>
+      <c r="I235" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J235" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K235" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L235" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M235" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="55" customHeight="1">
+      <c r="A236" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B236" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C236" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D236" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E236" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F236" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G236" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H236" s="146" t="inlineStr"/>
+      <c r="I236" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J236" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K236" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L236" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M236" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="55" customHeight="1">
+      <c r="A237" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B237" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C237" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D237" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E237" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F237" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G237" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H237" s="146" t="inlineStr"/>
+      <c r="I237" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J237" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K237" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L237" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M237" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="55" customHeight="1">
+      <c r="A238" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B238" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C238" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D238" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E238" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F238" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G238" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H238" s="146" t="inlineStr"/>
+      <c r="I238" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J238" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K238" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L238" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M238" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="55" customHeight="1">
+      <c r="A239" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B239" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C239" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D239" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E239" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F239" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G239" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H239" s="153" t="inlineStr"/>
+      <c r="I239" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J239" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K239" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L239" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M239" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="240" ht="55" customHeight="1">
+      <c r="A240" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B240" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C240" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D240" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E240" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F240" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G240" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H240" s="153" t="inlineStr"/>
+      <c r="I240" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J240" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K240" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L240" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M240" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" ht="55" customHeight="1">
+      <c r="A241" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B241" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent- Uppsala</t>
+        </is>
+      </c>
+      <c r="C241" s="152" t="inlineStr">
+        <is>
+          <t>Inova Assistans AB</t>
+        </is>
+      </c>
+      <c r="D241" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E241" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F241" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G241" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H241" s="153" t="inlineStr"/>
+      <c r="I241" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J241" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K241" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L241" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M241" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-31
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="242" ht="55" customHeight="1">
+      <c r="A242" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B242" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C242" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D242" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E242" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F242" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G242" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H242" s="153" t="inlineStr"/>
+      <c r="I242" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J242" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K242" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L242" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M242" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="243" ht="55" customHeight="1">
+      <c r="A243" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B243" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C243" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D243" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E243" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F243" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G243" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H243" s="153" t="inlineStr"/>
+      <c r="I243" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J243" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K243" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L243" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M243" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="244" ht="55" customHeight="1">
+      <c r="A244" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B244" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C244" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D244" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E244" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F244" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G244" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H244" s="153" t="inlineStr"/>
+      <c r="I244" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J244" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K244" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L244" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M244" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="245" ht="55" customHeight="1">
+      <c r="A245" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B245" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till aktiv man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C245" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D245" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E245" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F245" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G245" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H245" s="153" t="inlineStr"/>
+      <c r="I245" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J245" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K245" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L245" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M245" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="246" ht="55" customHeight="1">
+      <c r="A246" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B246" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C246" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D246" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E246" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F246" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G246" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H246" s="153" t="inlineStr"/>
+      <c r="I246" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J246" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K246" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L246" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M246" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="247" ht="55" customHeight="1">
+      <c r="A247" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B247" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C247" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D247" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E247" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F247" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G247" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H247" s="153" t="inlineStr"/>
+      <c r="I247" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J247" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K247" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L247" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M247" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
 🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
@@ -16508,6 +17431,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B231" r:id="rId191"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B232" r:id="rId192"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B233" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B234" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B235" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B236" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B237" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B238" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B239" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B240" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B241" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B242" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B243" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B244" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B245" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B246" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B247" r:id="rId207"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-07-08
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M247"/>
+  <dimension ref="A1:M249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-07 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-08 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -17224,6 +17224,137 @@
           <t>🆕 NYTT
 2026-02-19
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="248" ht="55" customHeight="1">
+      <c r="A248" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B248" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C248" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D248" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E248" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F248" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G248" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H248" s="153" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I248" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J248" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K248" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L248" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M248" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-07
+🏛️ Platsbanken #31256389</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="55" customHeight="1">
+      <c r="A249" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B249" s="129" t="inlineStr">
+        <is>
+          <t>NyPersonliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C249" s="152" t="inlineStr"/>
+      <c r="D249" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E249" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F249" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G249" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H249" s="153" t="inlineStr"/>
+      <c r="I249" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J249" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K249" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L249" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M249" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🔵 ledigajobb.se</t>
         </is>
       </c>
     </row>
@@ -17445,6 +17576,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B245" r:id="rId205"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B246" r:id="rId206"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B247" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B248" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B249" r:id="rId209"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-07-09
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M249"/>
+  <dimension ref="A1:M250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-08 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-09 · 8 källor · Radie &lt;50 km · 1 nya · 2 borttagna</t>
         </is>
       </c>
     </row>
@@ -17355,6 +17355,76 @@
         <is>
           <t>🆕 NYTT
 🔵 ledigajobb.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="250" ht="55" customHeight="1">
+      <c r="A250" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B250" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C250" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D250" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E250" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F250" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G250" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H250" s="153" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I250" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J250" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K250" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L250" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M250" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-08
+🏛️ Platsbanken #31257193</t>
         </is>
       </c>
     </row>
@@ -17578,6 +17648,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B247" r:id="rId207"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B248" r:id="rId208"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B249" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B250" r:id="rId210"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-07-13
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M250"/>
+  <dimension ref="A1:M263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-12 · 8 källor · Radie &lt;50 km · 0 nya · 13 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-13 · 8 källor · Radie &lt;50 km · 13 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -17425,6 +17425,863 @@
           <t>🆕 NYTT
 2026-07-08
 🏛️ Platsbanken #31257193</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" ht="55" customHeight="1">
+      <c r="A251" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B251" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C251" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D251" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E251" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F251" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G251" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H251" s="146" t="inlineStr"/>
+      <c r="I251" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J251" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K251" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L251" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M251" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="252" ht="55" customHeight="1">
+      <c r="A252" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B252" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C252" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D252" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E252" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F252" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G252" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H252" s="146" t="inlineStr"/>
+      <c r="I252" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J252" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K252" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L252" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M252" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" ht="55" customHeight="1">
+      <c r="A253" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B253" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C253" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D253" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E253" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F253" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G253" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H253" s="146" t="inlineStr"/>
+      <c r="I253" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J253" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K253" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L253" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M253" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" ht="55" customHeight="1">
+      <c r="A254" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B254" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C254" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D254" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E254" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F254" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G254" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H254" s="146" t="inlineStr"/>
+      <c r="I254" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J254" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K254" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L254" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M254" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" ht="55" customHeight="1">
+      <c r="A255" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B255" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C255" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D255" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E255" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F255" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G255" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H255" s="146" t="inlineStr"/>
+      <c r="I255" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J255" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K255" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L255" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M255" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="256" ht="55" customHeight="1">
+      <c r="A256" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B256" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C256" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D256" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E256" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F256" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G256" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H256" s="153" t="inlineStr"/>
+      <c r="I256" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J256" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K256" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L256" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M256" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="257" ht="55" customHeight="1">
+      <c r="A257" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B257" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C257" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D257" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E257" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F257" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G257" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H257" s="153" t="inlineStr"/>
+      <c r="I257" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J257" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K257" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L257" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M257" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="258" ht="55" customHeight="1">
+      <c r="A258" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B258" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C258" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D258" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E258" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F258" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G258" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H258" s="153" t="inlineStr"/>
+      <c r="I258" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J258" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K258" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L258" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M258" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" ht="55" customHeight="1">
+      <c r="A259" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B259" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C259" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D259" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E259" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F259" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G259" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H259" s="153" t="inlineStr"/>
+      <c r="I259" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J259" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K259" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L259" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M259" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" ht="55" customHeight="1">
+      <c r="A260" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B260" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C260" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D260" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E260" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F260" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G260" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H260" s="153" t="inlineStr"/>
+      <c r="I260" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J260" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K260" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L260" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M260" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="261" ht="55" customHeight="1">
+      <c r="A261" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B261" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till aktiv man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C261" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D261" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E261" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F261" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G261" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H261" s="153" t="inlineStr"/>
+      <c r="I261" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J261" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K261" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L261" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M261" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="262" ht="55" customHeight="1">
+      <c r="A262" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B262" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C262" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D262" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E262" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F262" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G262" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H262" s="153" t="inlineStr"/>
+      <c r="I262" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J262" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K262" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L262" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M262" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" ht="55" customHeight="1">
+      <c r="A263" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B263" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C263" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D263" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E263" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F263" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G263" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H263" s="153" t="inlineStr"/>
+      <c r="I263" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J263" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K263" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L263" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M263" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -17649,6 +18506,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B248" r:id="rId208"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B249" r:id="rId209"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B250" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B251" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B252" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B253" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B254" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B255" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B256" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B257" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B258" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B259" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B260" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B261" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B262" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B263" r:id="rId223"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-07-18
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M263"/>
+  <dimension ref="A1:M279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-17 · 8 källor · Radie &lt;50 km · 0 nya · 13 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-18 · 8 källor · Radie &lt;50 km · 16 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -18278,6 +18278,1069 @@
         </is>
       </c>
       <c r="M263" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="264" ht="55" customHeight="1">
+      <c r="A264" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B264" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C264" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D264" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E264" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F264" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G264" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H264" s="146" t="inlineStr"/>
+      <c r="I264" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J264" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K264" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L264" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M264" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="265" ht="55" customHeight="1">
+      <c r="A265" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B265" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C265" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D265" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E265" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F265" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G265" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H265" s="146" t="inlineStr"/>
+      <c r="I265" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J265" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K265" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L265" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M265" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="266" ht="55" customHeight="1">
+      <c r="A266" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B266" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C266" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D266" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E266" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F266" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G266" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H266" s="146" t="inlineStr"/>
+      <c r="I266" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J266" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K266" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L266" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M266" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="267" ht="55" customHeight="1">
+      <c r="A267" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B267" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C267" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D267" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E267" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F267" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G267" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H267" s="146" t="inlineStr"/>
+      <c r="I267" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J267" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K267" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L267" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M267" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="268" ht="55" customHeight="1">
+      <c r="A268" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B268" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C268" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D268" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E268" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F268" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G268" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H268" s="146" t="inlineStr"/>
+      <c r="I268" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J268" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K268" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L268" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M268" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="269" ht="55" customHeight="1">
+      <c r="A269" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B269" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C269" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D269" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E269" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F269" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G269" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H269" s="146" t="inlineStr"/>
+      <c r="I269" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J269" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K269" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L269" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M269" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="270" ht="55" customHeight="1">
+      <c r="A270" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B270" s="129" t="inlineStr">
+        <is>
+          <t>Gillar du att hitta på roliga saker med en kille i Tobo/Örbyhus?</t>
+        </is>
+      </c>
+      <c r="C270" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D270" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E270" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F270" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G270" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H270" s="153" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I270" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J270" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K270" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L270" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M270" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-17
+🏛️ Platsbanken #31280379</t>
+        </is>
+      </c>
+    </row>
+    <row r="271" ht="55" customHeight="1">
+      <c r="A271" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B271" s="129" t="inlineStr">
+        <is>
+          <t>Assistent sökes till 32-årig mjukvaruutvecklare i Uppsala, ca 70%</t>
+        </is>
+      </c>
+      <c r="C271" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D271" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E271" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F271" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G271" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H271" s="153" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="I271" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J271" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K271" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L271" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M271" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-17
+🏛️ Platsbanken #31280243</t>
+        </is>
+      </c>
+    </row>
+    <row r="272" ht="55" customHeight="1">
+      <c r="A272" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B272" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C272" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D272" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E272" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F272" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G272" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H272" s="153" t="inlineStr"/>
+      <c r="I272" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J272" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K272" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L272" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M272" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="273" ht="55" customHeight="1">
+      <c r="A273" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B273" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C273" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D273" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E273" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F273" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G273" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H273" s="153" t="inlineStr"/>
+      <c r="I273" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J273" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K273" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L273" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M273" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="274" ht="55" customHeight="1">
+      <c r="A274" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B274" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C274" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D274" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E274" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F274" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G274" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H274" s="153" t="inlineStr"/>
+      <c r="I274" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J274" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K274" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L274" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M274" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="275" ht="55" customHeight="1">
+      <c r="A275" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B275" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C275" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D275" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E275" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F275" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G275" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H275" s="153" t="inlineStr"/>
+      <c r="I275" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J275" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K275" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L275" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M275" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="276" ht="55" customHeight="1">
+      <c r="A276" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B276" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C276" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D276" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E276" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F276" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G276" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H276" s="153" t="inlineStr"/>
+      <c r="I276" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J276" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K276" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L276" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M276" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="277" ht="55" customHeight="1">
+      <c r="A277" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B277" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till aktiv man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C277" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D277" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E277" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F277" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G277" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H277" s="153" t="inlineStr"/>
+      <c r="I277" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J277" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K277" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L277" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M277" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="278" ht="55" customHeight="1">
+      <c r="A278" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B278" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C278" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D278" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E278" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F278" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G278" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H278" s="153" t="inlineStr"/>
+      <c r="I278" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J278" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K278" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L278" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M278" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="279" ht="55" customHeight="1">
+      <c r="A279" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B279" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C279" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D279" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E279" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F279" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G279" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H279" s="153" t="inlineStr"/>
+      <c r="I279" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J279" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K279" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L279" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M279" s="154" t="inlineStr">
         <is>
           <t>🆕 NYTT
 2026-02-19
@@ -18519,6 +19582,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B261" r:id="rId221"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B262" r:id="rId222"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B263" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B264" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B265" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B266" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B267" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B268" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B269" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B270" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B271" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B272" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B273" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B274" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B275" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B276" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B277" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B278" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B279" r:id="rId239"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-07-21
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M279"/>
+  <dimension ref="A1:M280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-19 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-21 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -19345,6 +19345,76 @@
           <t>🆕 NYTT
 2026-02-19
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="280" ht="55" customHeight="1">
+      <c r="A280" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B280" s="129" t="inlineStr">
+        <is>
+          <t>Spännade assistansjobb utanför Uppsala till en man.</t>
+        </is>
+      </c>
+      <c r="C280" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D280" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E280" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F280" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G280" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H280" s="153" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="I280" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J280" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K280" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L280" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M280" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-20
+🏛️ Platsbanken #31283307</t>
         </is>
       </c>
     </row>
@@ -19598,6 +19668,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B277" r:id="rId237"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B278" r:id="rId238"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B279" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B280" r:id="rId240"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-07-23
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M280"/>
+  <dimension ref="A1:M282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-21 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-23 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -19415,6 +19415,148 @@
           <t>🆕 NYTT
 2026-07-20
 🏛️ Platsbanken #31283307</t>
+        </is>
+      </c>
+    </row>
+    <row r="281" ht="55" customHeight="1">
+      <c r="A281" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B281" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till man i centrala Uppsala (deltid och vikarietjänst)</t>
+        </is>
+      </c>
+      <c r="C281" s="152" t="inlineStr">
+        <is>
+          <t>JAG Personlig assistans</t>
+        </is>
+      </c>
+      <c r="D281" s="152" t="inlineStr">
+        <is>
+          <t>deltid och vikarietjänst) Deltid ,
+ tills vidare,
+ varaktighet: vanlig anställning JAG Personlig assistans (Uppsala</t>
+        </is>
+      </c>
+      <c r="E281" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F281" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G281" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H281" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="I281" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J281" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K281" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L281" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M281" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-22
+🏛️ Platsbanken #31288239</t>
+        </is>
+      </c>
+    </row>
+    <row r="282" ht="55" customHeight="1">
+      <c r="A282" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B282" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till en ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C282" s="152" t="inlineStr">
+        <is>
+          <t>Särnmark Assistans AB</t>
+        </is>
+      </c>
+      <c r="D282" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E282" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F282" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G282" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H282" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="I282" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J282" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K282" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L282" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M282" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-22
+🏛️ Platsbanken #31287757</t>
         </is>
       </c>
     </row>
@@ -19669,6 +19811,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B278" r:id="rId238"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B279" r:id="rId239"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B280" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B281" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B282" r:id="rId242"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-07-28
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M282"/>
+  <dimension ref="A1:M283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-24 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-28 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -19557,6 +19557,76 @@
           <t>🆕 NYTT
 2026-07-22
 🏛️ Platsbanken #31287757</t>
+        </is>
+      </c>
+    </row>
+    <row r="283" ht="55" customHeight="1">
+      <c r="A283" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B283" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till en 9-årig pojke – 30–50 %</t>
+        </is>
+      </c>
+      <c r="C283" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D283" s="157" t="inlineStr">
+        <is>
+          <t>Tierp</t>
+        </is>
+      </c>
+      <c r="E283" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F283" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G283" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H283" s="158" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="I283" s="158" t="inlineStr">
+        <is>
+          <t>~43 km</t>
+        </is>
+      </c>
+      <c r="J283" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K283" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L283" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M283" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-27
+🏛️ Platsbanken #31297045</t>
         </is>
       </c>
     </row>
@@ -19813,6 +19883,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B280" r:id="rId240"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B281" r:id="rId241"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B282" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B283" r:id="rId243"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-07-31
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M283"/>
+  <dimension ref="A1:M298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-30 · 8 källor · Radie &lt;50 km · 0 nya · 14 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-07-31 · 8 källor · Radie &lt;50 km · 15 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -19627,6 +19627,999 @@
           <t>🆕 NYTT
 2026-07-27
 🏛️ Platsbanken #31297045</t>
+        </is>
+      </c>
+    </row>
+    <row r="284" ht="55" customHeight="1">
+      <c r="A284" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B284" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C284" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D284" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E284" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F284" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G284" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H284" s="146" t="inlineStr"/>
+      <c r="I284" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J284" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K284" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L284" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M284" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="285" ht="55" customHeight="1">
+      <c r="A285" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B285" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C285" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D285" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E285" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F285" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G285" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H285" s="146" t="inlineStr"/>
+      <c r="I285" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J285" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K285" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L285" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M285" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="286" ht="55" customHeight="1">
+      <c r="A286" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B286" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C286" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D286" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E286" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F286" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G286" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H286" s="146" t="inlineStr"/>
+      <c r="I286" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J286" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K286" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L286" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M286" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="287" ht="55" customHeight="1">
+      <c r="A287" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B287" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C287" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D287" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E287" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F287" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G287" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H287" s="146" t="inlineStr"/>
+      <c r="I287" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J287" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K287" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L287" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M287" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="288" ht="55" customHeight="1">
+      <c r="A288" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B288" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C288" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D288" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E288" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F288" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G288" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H288" s="146" t="inlineStr"/>
+      <c r="I288" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J288" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K288" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L288" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M288" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="289" ht="55" customHeight="1">
+      <c r="A289" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B289" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C289" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D289" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E289" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F289" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G289" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H289" s="146" t="inlineStr"/>
+      <c r="I289" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J289" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K289" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L289" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M289" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="290" ht="55" customHeight="1">
+      <c r="A290" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B290" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C290" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D290" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E290" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F290" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G290" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H290" s="153" t="inlineStr"/>
+      <c r="I290" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J290" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K290" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L290" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M290" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="291" ht="55" customHeight="1">
+      <c r="A291" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B291" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C291" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D291" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E291" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F291" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G291" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H291" s="153" t="inlineStr"/>
+      <c r="I291" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J291" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K291" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L291" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M291" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="292" ht="55" customHeight="1">
+      <c r="A292" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B292" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C292" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D292" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E292" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F292" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G292" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H292" s="153" t="inlineStr"/>
+      <c r="I292" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J292" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K292" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L292" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M292" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="293" ht="55" customHeight="1">
+      <c r="A293" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B293" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C293" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D293" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E293" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F293" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G293" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H293" s="153" t="inlineStr"/>
+      <c r="I293" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J293" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K293" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L293" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M293" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="294" ht="55" customHeight="1">
+      <c r="A294" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B294" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C294" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D294" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E294" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F294" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G294" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H294" s="153" t="inlineStr"/>
+      <c r="I294" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J294" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K294" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L294" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M294" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="295" ht="55" customHeight="1">
+      <c r="A295" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B295" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till aktiv man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C295" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D295" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E295" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F295" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G295" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H295" s="153" t="inlineStr"/>
+      <c r="I295" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J295" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K295" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L295" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M295" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="296" ht="55" customHeight="1">
+      <c r="A296" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B296" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C296" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D296" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E296" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F296" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G296" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H296" s="153" t="inlineStr"/>
+      <c r="I296" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J296" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K296" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L296" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M296" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="297" ht="55" customHeight="1">
+      <c r="A297" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B297" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C297" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D297" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E297" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F297" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G297" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H297" s="153" t="inlineStr"/>
+      <c r="I297" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J297" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K297" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L297" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M297" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="298" ht="55" customHeight="1">
+      <c r="A298" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B298" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent, timvikariat, sökes till man i Heby</t>
+        </is>
+      </c>
+      <c r="C298" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D298" s="157" t="inlineStr">
+        <is>
+          <t>Heby</t>
+        </is>
+      </c>
+      <c r="E298" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F298" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G298" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H298" s="158" t="inlineStr">
+        <is>
+          <t>2027-01-26</t>
+        </is>
+      </c>
+      <c r="I298" s="158" t="inlineStr">
+        <is>
+          <t>~47 km</t>
+        </is>
+      </c>
+      <c r="J298" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K298" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L298" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M298" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-30
+🏛️ Platsbanken #31305031</t>
         </is>
       </c>
     </row>
@@ -19884,6 +20877,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B281" r:id="rId241"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B282" r:id="rId242"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B283" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B284" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B285" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B286" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B287" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B288" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B289" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B290" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B291" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B292" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B293" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B294" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B295" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B296" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B297" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B298" r:id="rId258"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-04
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M298"/>
+  <dimension ref="A1:M312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-03 · 8 källor · Radie &lt;50 km · 0 nya · 14 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-04 · 8 källor · Radie &lt;50 km · 14 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -20620,6 +20620,929 @@
           <t>🆕 NYTT
 2026-07-30
 🏛️ Platsbanken #31305031</t>
+        </is>
+      </c>
+    </row>
+    <row r="299" ht="55" customHeight="1">
+      <c r="A299" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B299" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C299" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D299" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E299" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F299" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G299" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H299" s="146" t="inlineStr"/>
+      <c r="I299" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J299" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K299" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L299" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M299" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="300" ht="55" customHeight="1">
+      <c r="A300" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B300" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C300" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D300" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E300" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F300" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G300" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H300" s="146" t="inlineStr"/>
+      <c r="I300" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J300" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K300" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L300" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M300" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="55" customHeight="1">
+      <c r="A301" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B301" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C301" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D301" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E301" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F301" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G301" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H301" s="146" t="inlineStr"/>
+      <c r="I301" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J301" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K301" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L301" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M301" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="302" ht="55" customHeight="1">
+      <c r="A302" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B302" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C302" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D302" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E302" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F302" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G302" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H302" s="146" t="inlineStr"/>
+      <c r="I302" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J302" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K302" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L302" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M302" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="303" ht="55" customHeight="1">
+      <c r="A303" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B303" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C303" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D303" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E303" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F303" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G303" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H303" s="146" t="inlineStr"/>
+      <c r="I303" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J303" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K303" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L303" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M303" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="304" ht="55" customHeight="1">
+      <c r="A304" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B304" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C304" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D304" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E304" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F304" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G304" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H304" s="146" t="inlineStr"/>
+      <c r="I304" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J304" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K304" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L304" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M304" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="305" ht="55" customHeight="1">
+      <c r="A305" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B305" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C305" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D305" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E305" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F305" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G305" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H305" s="153" t="inlineStr"/>
+      <c r="I305" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J305" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K305" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L305" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M305" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="306" ht="55" customHeight="1">
+      <c r="A306" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B306" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C306" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D306" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E306" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F306" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G306" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H306" s="153" t="inlineStr"/>
+      <c r="I306" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J306" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K306" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L306" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M306" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="307" ht="55" customHeight="1">
+      <c r="A307" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B307" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C307" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D307" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E307" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F307" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G307" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H307" s="153" t="inlineStr"/>
+      <c r="I307" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J307" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K307" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L307" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M307" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="308" ht="55" customHeight="1">
+      <c r="A308" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B308" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C308" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D308" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E308" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F308" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G308" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H308" s="153" t="inlineStr"/>
+      <c r="I308" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J308" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K308" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L308" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M308" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="309" ht="55" customHeight="1">
+      <c r="A309" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B309" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C309" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D309" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E309" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F309" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G309" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H309" s="153" t="inlineStr"/>
+      <c r="I309" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J309" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K309" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L309" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M309" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" ht="55" customHeight="1">
+      <c r="A310" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B310" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till aktiv man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C310" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D310" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E310" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F310" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G310" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H310" s="153" t="inlineStr"/>
+      <c r="I310" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J310" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K310" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L310" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M310" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="55" customHeight="1">
+      <c r="A311" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B311" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C311" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D311" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E311" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F311" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G311" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H311" s="153" t="inlineStr"/>
+      <c r="I311" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J311" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K311" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L311" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M311" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="55" customHeight="1">
+      <c r="A312" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B312" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C312" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D312" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E312" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F312" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G312" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H312" s="153" t="inlineStr"/>
+      <c r="I312" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J312" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K312" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L312" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M312" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -20892,6 +21815,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B296" r:id="rId256"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B297" r:id="rId257"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B298" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B299" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B300" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B301" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B302" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B303" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B304" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B305" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B306" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B307" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B308" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B309" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B310" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B311" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B312" r:id="rId272"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-06
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M312"/>
+  <dimension ref="A1:M314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-04 · 8 källor · Radie &lt;50 km · 14 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-06 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -21542,6 +21542,142 @@
         <is>
           <t>🆕 NYTT
 2026-02-19
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="313" ht="55" customHeight="1">
+      <c r="A313" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B313" s="129" t="inlineStr">
+        <is>
+          <t>Assistent med körkort sökes till kille</t>
+        </is>
+      </c>
+      <c r="C313" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D313" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E313" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F313" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G313" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H313" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="I313" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J313" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K313" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L313" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M313" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-05
+🏛️ Platsbanken #31321002</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="55" customHeight="1">
+      <c r="A314" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B314" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent- Uppsala</t>
+        </is>
+      </c>
+      <c r="C314" s="152" t="inlineStr">
+        <is>
+          <t>Inova Assistans AB</t>
+        </is>
+      </c>
+      <c r="D314" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E314" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F314" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G314" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H314" s="153" t="inlineStr"/>
+      <c r="I314" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J314" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K314" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L314" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M314" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-31
 🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
@@ -21829,6 +21965,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B310" r:id="rId270"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B311" r:id="rId271"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B312" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B313" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B314" r:id="rId274"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-07
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M314"/>
+  <dimension ref="A1:M315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-06 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-07 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -21679,6 +21679,76 @@
           <t>🆕 NYTT
 2026-03-31
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="315" ht="55" customHeight="1">
+      <c r="A315" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B315" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till en man i Bålsta</t>
+        </is>
+      </c>
+      <c r="C315" s="152" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="D315" s="152" t="inlineStr">
+        <is>
+          <t>Håbo</t>
+        </is>
+      </c>
+      <c r="E315" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F315" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G315" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H315" s="153" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="I315" s="153" t="inlineStr">
+        <is>
+          <t>~45 km</t>
+        </is>
+      </c>
+      <c r="J315" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K315" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L315" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Diskutera semester.</t>
+        </is>
+      </c>
+      <c r="M315" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-06
+🏛️ Platsbanken #31325036</t>
         </is>
       </c>
     </row>
@@ -21967,6 +22037,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B312" r:id="rId272"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B313" r:id="rId273"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B314" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B315" r:id="rId275"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-08
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M315"/>
+  <dimension ref="A1:M316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-07 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-08 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -21749,6 +21749,76 @@
           <t>🆕 NYTT
 2026-08-06
 🏛️ Platsbanken #31325036</t>
+        </is>
+      </c>
+    </row>
+    <row r="316" ht="55" customHeight="1">
+      <c r="A316" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B316" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent sökes till man i Uppsala - fast schemarad</t>
+        </is>
+      </c>
+      <c r="C316" s="152" t="inlineStr">
+        <is>
+          <t>Livsam Personlig Assistans AB</t>
+        </is>
+      </c>
+      <c r="D316" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E316" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F316" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G316" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H316" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I316" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J316" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K316" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L316" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M316" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-07
+🏛️ Platsbanken #31328443</t>
         </is>
       </c>
     </row>
@@ -22038,6 +22108,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B313" r:id="rId273"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B314" r:id="rId274"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B315" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B316" r:id="rId276"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-12
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M316"/>
+  <dimension ref="A1:M317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-08 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-12 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -21819,6 +21819,76 @@
           <t>🆕 NYTT
 2026-08-07
 🏛️ Platsbanken #31328443</t>
+        </is>
+      </c>
+    </row>
+    <row r="317" ht="55" customHeight="1">
+      <c r="A317" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B317" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till kille mellan Månkarbo och Östervåla</t>
+        </is>
+      </c>
+      <c r="C317" s="152" t="inlineStr">
+        <is>
+          <t>Särnmark Assistans AB</t>
+        </is>
+      </c>
+      <c r="D317" s="152" t="inlineStr">
+        <is>
+          <t>Heby</t>
+        </is>
+      </c>
+      <c r="E317" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F317" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G317" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H317" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="I317" s="153" t="inlineStr">
+        <is>
+          <t>~47 km</t>
+        </is>
+      </c>
+      <c r="J317" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K317" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L317" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M317" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-11
+🏛️ Platsbanken #31338899</t>
         </is>
       </c>
     </row>
@@ -22109,6 +22179,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B314" r:id="rId274"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B315" r:id="rId275"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B316" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B317" r:id="rId277"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-13
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M317"/>
+  <dimension ref="A1:M319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-12 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-13 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -21889,6 +21889,146 @@
           <t>🆕 NYTT
 2026-08-11
 🏛️ Platsbanken #31338899</t>
+        </is>
+      </c>
+    </row>
+    <row r="318" ht="55" customHeight="1">
+      <c r="A318" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B318" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig som vill arbeta som personlig assistent åt en trevlig 62-årig Man</t>
+        </is>
+      </c>
+      <c r="C318" s="152" t="inlineStr">
+        <is>
+          <t>Assistans i Balans i Sverige AB</t>
+        </is>
+      </c>
+      <c r="D318" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E318" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F318" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G318" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H318" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="I318" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J318" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K318" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L318" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M318" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-12
+🏛️ Platsbanken #31345608</t>
+        </is>
+      </c>
+    </row>
+    <row r="319" ht="55" customHeight="1">
+      <c r="A319" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B319" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter sökes till kille utanför Uppsala</t>
+        </is>
+      </c>
+      <c r="C319" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D319" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E319" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F319" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G319" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H319" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="I319" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J319" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K319" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L319" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M319" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-12
+🏛️ Platsbanken #31343535</t>
         </is>
       </c>
     </row>
@@ -22180,6 +22320,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B315" r:id="rId275"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B316" r:id="rId276"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B317" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B318" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B319" r:id="rId279"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-14
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M319"/>
+  <dimension ref="A1:M320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-13 · 8 källor · Radie &lt;50 km · 2 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-14 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -22029,6 +22029,76 @@
           <t>🆕 NYTT
 2026-08-12
 🏛️ Platsbanken #31343535</t>
+        </is>
+      </c>
+    </row>
+    <row r="320" ht="55" customHeight="1">
+      <c r="A320" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B320" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till matlagningsintresserad man i Uppsla</t>
+        </is>
+      </c>
+      <c r="C320" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D320" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E320" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F320" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G320" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H320" s="153" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="I320" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J320" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K320" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L320" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M320" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-13
+🏛️ Platsbanken #31348037</t>
         </is>
       </c>
     </row>
@@ -22322,6 +22392,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B317" r:id="rId277"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B318" r:id="rId278"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B319" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B320" r:id="rId280"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-17
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M320"/>
+  <dimension ref="A1:M321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-14 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-17 · 8 källor · Radie &lt;50 km · 1 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -22099,6 +22099,76 @@
           <t>🆕 NYTT
 2026-08-13
 🏛️ Platsbanken #31348037</t>
+        </is>
+      </c>
+    </row>
+    <row r="321" ht="55" customHeight="1">
+      <c r="A321" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B321" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent  till 3-årig pojke i Uppsala</t>
+        </is>
+      </c>
+      <c r="C321" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D321" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E321" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F321" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G321" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H321" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="I321" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J321" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K321" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L321" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M321" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-16
+🏛️ Platsbanken #31356836</t>
         </is>
       </c>
     </row>
@@ -22393,6 +22463,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B318" r:id="rId278"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B319" r:id="rId279"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B320" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B321" r:id="rId281"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-19
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M321"/>
+  <dimension ref="A1:M336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-18 · 8 källor · Radie &lt;50 km · 0 nya · 15 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-19 · 8 källor · Radie &lt;50 km · 15 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -22169,6 +22169,995 @@
           <t>🆕 NYTT
 2026-08-16
 🏛️ Platsbanken #31356836</t>
+        </is>
+      </c>
+    </row>
+    <row r="322" ht="55" customHeight="1">
+      <c r="A322" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B322" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C322" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D322" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E322" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F322" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G322" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H322" s="146" t="inlineStr"/>
+      <c r="I322" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J322" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K322" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L322" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M322" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="323" ht="55" customHeight="1">
+      <c r="A323" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B323" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C323" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D323" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E323" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F323" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G323" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H323" s="146" t="inlineStr"/>
+      <c r="I323" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J323" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K323" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L323" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M323" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="324" ht="55" customHeight="1">
+      <c r="A324" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B324" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C324" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D324" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E324" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F324" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G324" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H324" s="146" t="inlineStr"/>
+      <c r="I324" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J324" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K324" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L324" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M324" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="325" ht="55" customHeight="1">
+      <c r="A325" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B325" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C325" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D325" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E325" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F325" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G325" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H325" s="146" t="inlineStr"/>
+      <c r="I325" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J325" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K325" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L325" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M325" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="326" ht="55" customHeight="1">
+      <c r="A326" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B326" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C326" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D326" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E326" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F326" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G326" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H326" s="146" t="inlineStr"/>
+      <c r="I326" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J326" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K326" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L326" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M326" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="327" ht="55" customHeight="1">
+      <c r="A327" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B327" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C327" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D327" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E327" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F327" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G327" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H327" s="146" t="inlineStr"/>
+      <c r="I327" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J327" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K327" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L327" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M327" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="328" ht="55" customHeight="1">
+      <c r="A328" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B328" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C328" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D328" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E328" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F328" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G328" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H328" s="153" t="inlineStr"/>
+      <c r="I328" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J328" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K328" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L328" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M328" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="329" ht="55" customHeight="1">
+      <c r="A329" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B329" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C329" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D329" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E329" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F329" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G329" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H329" s="153" t="inlineStr"/>
+      <c r="I329" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J329" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K329" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L329" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M329" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="330" ht="55" customHeight="1">
+      <c r="A330" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B330" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent- Uppsala</t>
+        </is>
+      </c>
+      <c r="C330" s="152" t="inlineStr">
+        <is>
+          <t>Inova Assistans AB</t>
+        </is>
+      </c>
+      <c r="D330" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E330" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F330" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G330" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H330" s="153" t="inlineStr"/>
+      <c r="I330" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J330" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K330" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L330" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M330" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-31
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="331" ht="55" customHeight="1">
+      <c r="A331" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B331" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C331" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D331" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E331" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F331" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G331" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H331" s="153" t="inlineStr"/>
+      <c r="I331" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J331" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K331" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L331" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M331" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="55" customHeight="1">
+      <c r="A332" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B332" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C332" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D332" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E332" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F332" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G332" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H332" s="153" t="inlineStr"/>
+      <c r="I332" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J332" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K332" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L332" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M332" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="333" ht="55" customHeight="1">
+      <c r="A333" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B333" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C333" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D333" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E333" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F333" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G333" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H333" s="153" t="inlineStr"/>
+      <c r="I333" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J333" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K333" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L333" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M333" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="334" ht="55" customHeight="1">
+      <c r="A334" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B334" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till aktiv man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C334" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D334" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E334" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F334" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G334" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H334" s="153" t="inlineStr"/>
+      <c r="I334" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J334" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K334" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L334" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M334" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="335" ht="55" customHeight="1">
+      <c r="A335" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B335" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C335" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D335" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E335" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F335" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G335" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H335" s="153" t="inlineStr"/>
+      <c r="I335" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J335" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K335" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L335" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M335" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="336" ht="55" customHeight="1">
+      <c r="A336" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B336" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C336" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D336" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E336" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F336" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G336" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H336" s="153" t="inlineStr"/>
+      <c r="I336" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J336" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K336" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L336" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M336" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -22464,6 +23453,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B319" r:id="rId279"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B320" r:id="rId280"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B321" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B322" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B323" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B324" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B325" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B326" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B327" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B328" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B329" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B330" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B331" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B332" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B333" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B334" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B335" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B336" r:id="rId296"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-20
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M336"/>
+  <dimension ref="A1:M338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-19 · 8 källor · Radie &lt;50 km · 15 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-20 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -23158,6 +23158,142 @@
           <t>🆕 NYTT
 2026-02-19
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="55" customHeight="1">
+      <c r="A337" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B337" s="123" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C337" s="145" t="inlineStr">
+        <is>
+          <t>Inkludera assistans i Sverige AB</t>
+        </is>
+      </c>
+      <c r="D337" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E337" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F337" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G337" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H337" s="146" t="inlineStr"/>
+      <c r="I337" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J337" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K337" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L337" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M337" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="55" customHeight="1">
+      <c r="A338" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B338" s="133" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till matlagningsintresserad man i Tierp</t>
+        </is>
+      </c>
+      <c r="C338" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D338" s="157" t="inlineStr">
+        <is>
+          <t>Tierp</t>
+        </is>
+      </c>
+      <c r="E338" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F338" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G338" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H338" s="158" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="I338" s="158" t="inlineStr">
+        <is>
+          <t>~43 km</t>
+        </is>
+      </c>
+      <c r="J338" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K338" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L338" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M338" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-19
+🏛️ Platsbanken #31370224</t>
         </is>
       </c>
     </row>
@@ -23468,6 +23604,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B334" r:id="rId294"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B335" r:id="rId295"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B336" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B337" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B338" r:id="rId298"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-21
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M338"/>
+  <dimension ref="A1:M339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-20 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-21 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -23294,6 +23294,76 @@
           <t>🆕 NYTT
 2026-08-19
 🏛️ Platsbanken #31370224</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="55" customHeight="1">
+      <c r="A339" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B339" s="133" t="inlineStr">
+        <is>
+          <t>Trygg och lyhörd assistent sökes till man i Tierp - vikariat</t>
+        </is>
+      </c>
+      <c r="C339" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D339" s="157" t="inlineStr">
+        <is>
+          <t>Tierp</t>
+        </is>
+      </c>
+      <c r="E339" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F339" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G339" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H339" s="158" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="I339" s="158" t="inlineStr">
+        <is>
+          <t>~43 km</t>
+        </is>
+      </c>
+      <c r="J339" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K339" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L339" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M339" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-20
+🏛️ Platsbanken #31375440</t>
         </is>
       </c>
     </row>
@@ -23606,6 +23676,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B336" r:id="rId296"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B337" r:id="rId297"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B338" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B339" r:id="rId299"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-22
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M339"/>
+  <dimension ref="A1:M340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-21 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-22 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -23364,6 +23364,76 @@
           <t>🆕 NYTT
 2026-08-20
 🏛️ Platsbanken #31375440</t>
+        </is>
+      </c>
+    </row>
+    <row r="340" ht="55" customHeight="1">
+      <c r="A340" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B340" s="129" t="inlineStr">
+        <is>
+          <t>Timanställd personlig assistent sökes till en kille Norrtälje/Uppsala!</t>
+        </is>
+      </c>
+      <c r="C340" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D340" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E340" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F340" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G340" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H340" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="I340" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J340" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K340" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L340" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M340" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-21
+🏛️ Platsbanken #31381141</t>
         </is>
       </c>
     </row>
@@ -23677,6 +23747,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B337" r:id="rId297"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B338" r:id="rId298"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B339" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B340" r:id="rId300"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-25
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M340"/>
+  <dimension ref="A1:M341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-23 · 8 källor · Radie &lt;50 km · 0 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-25 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -23434,6 +23434,76 @@
           <t>🆕 NYTT
 2026-08-21
 🏛️ Platsbanken #31381141</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="55" customHeight="1">
+      <c r="A341" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B341" s="129" t="inlineStr">
+        <is>
+          <t>Assistent till vuxen man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C341" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D341" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E341" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F341" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G341" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H341" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I341" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J341" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K341" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L341" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M341" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-24
+🏛️ Platsbanken #31389633</t>
         </is>
       </c>
     </row>
@@ -23748,6 +23818,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B338" r:id="rId298"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B339" r:id="rId299"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B340" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B341" r:id="rId301"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-26
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M341"/>
+  <dimension ref="A1:M343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-25 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-26 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -23504,6 +23504,146 @@
           <t>🆕 NYTT
 2026-08-24
 🏛️ Platsbanken #31389633</t>
+        </is>
+      </c>
+    </row>
+    <row r="342" ht="55" customHeight="1">
+      <c r="A342" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B342" s="129" t="inlineStr">
+        <is>
+          <t>Manlig assistent sökes till konst/Kultur intresserad man i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C342" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D342" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E342" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F342" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G342" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H342" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="I342" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J342" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K342" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L342" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M342" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-25
+🏛️ Platsbanken #31393596</t>
+        </is>
+      </c>
+    </row>
+    <row r="343" ht="55" customHeight="1">
+      <c r="A343" s="156" t="inlineStr">
+        <is>
+          <t>🆕 ⭐</t>
+        </is>
+      </c>
+      <c r="B343" s="133" t="inlineStr">
+        <is>
+          <t>Personlig assistent, timvikariat, sökes till man i Heby</t>
+        </is>
+      </c>
+      <c r="C343" s="157" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D343" s="157" t="inlineStr">
+        <is>
+          <t>Heby</t>
+        </is>
+      </c>
+      <c r="E343" s="157" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F343" s="157" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G343" s="158" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H343" s="158" t="inlineStr">
+        <is>
+          <t>2027-02-21</t>
+        </is>
+      </c>
+      <c r="I343" s="158" t="inlineStr">
+        <is>
+          <t>~47 km</t>
+        </is>
+      </c>
+      <c r="J343" s="157" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K343" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L343" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M343" s="160" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-25
+🏛️ Platsbanken #31394627</t>
         </is>
       </c>
     </row>
@@ -23819,6 +23959,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B339" r:id="rId299"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B340" r:id="rId300"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B341" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B342" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B343" r:id="rId303"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-27
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M343"/>
+  <dimension ref="A1:M345"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-26 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-27 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -23644,6 +23644,146 @@
           <t>🆕 NYTT
 2026-08-25
 🏛️ Platsbanken #31394627</t>
+        </is>
+      </c>
+    </row>
+    <row r="344" ht="55" customHeight="1">
+      <c r="A344" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B344" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarier sökes till social man i 70-års åldern i Uppsala</t>
+        </is>
+      </c>
+      <c r="C344" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D344" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E344" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F344" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G344" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H344" s="153" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="I344" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J344" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K344" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L344" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M344" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-26
+🏛️ Platsbanken #31401063</t>
+        </is>
+      </c>
+    </row>
+    <row r="345" ht="55" customHeight="1">
+      <c r="A345" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B345" s="129" t="inlineStr">
+        <is>
+          <t>Timvikarie sökes till aktiv man i centrala Uppsala</t>
+        </is>
+      </c>
+      <c r="C345" s="152" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D345" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E345" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F345" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G345" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H345" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="I345" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J345" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K345" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L345" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M345" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-26
+🏛️ Platsbanken #31398665</t>
         </is>
       </c>
     </row>
@@ -23961,6 +24101,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B341" r:id="rId301"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B342" r:id="rId302"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B343" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B344" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B345" r:id="rId305"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-28
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M345"/>
+  <dimension ref="A1:M346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-27 · 8 källor · Radie &lt;50 km · 2 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-28 · 8 källor · Radie &lt;50 km · 1 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -23784,6 +23784,76 @@
           <t>🆕 NYTT
 2026-08-26
 🏛️ Platsbanken #31398665</t>
+        </is>
+      </c>
+    </row>
+    <row r="346" ht="55" customHeight="1">
+      <c r="A346" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B346" s="129" t="inlineStr">
+        <is>
+          <t>vi söker dig som vill bli stödfamilj åt en 9-årig kille</t>
+        </is>
+      </c>
+      <c r="C346" s="152" t="inlineStr">
+        <is>
+          <t>Knivsta kommun</t>
+        </is>
+      </c>
+      <c r="D346" s="152" t="inlineStr">
+        <is>
+          <t>Knivsta</t>
+        </is>
+      </c>
+      <c r="E346" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F346" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G346" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H346" s="153" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="I346" s="153" t="inlineStr">
+        <is>
+          <t>~27 km</t>
+        </is>
+      </c>
+      <c r="J346" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K346" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L346" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Diskutera semester.</t>
+        </is>
+      </c>
+      <c r="M346" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-08-28
+🏛️ Platsbanken #31411141</t>
         </is>
       </c>
     </row>
@@ -24103,6 +24173,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B343" r:id="rId303"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B344" r:id="rId304"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B345" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B346" r:id="rId306"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-08-31
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M346"/>
+  <dimension ref="A1:M361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-29 · 8 källor · Radie &lt;50 km · 0 nya · 16 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-31 · 8 källor · Radie &lt;50 km · 15 nya · 1 borttagna</t>
         </is>
       </c>
     </row>
@@ -23854,6 +23854,995 @@
           <t>🆕 NYTT
 2026-08-28
 🏛️ Platsbanken #31411141</t>
+        </is>
+      </c>
+    </row>
+    <row r="347" ht="55" customHeight="1">
+      <c r="A347" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B347" s="123" t="inlineStr">
+        <is>
+          <t>Personliga assistenter till en kille i Uppsala.</t>
+        </is>
+      </c>
+      <c r="C347" s="145" t="inlineStr">
+        <is>
+          <t>Inkludera assistans i Sverige AB</t>
+        </is>
+      </c>
+      <c r="D347" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E347" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F347" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G347" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H347" s="146" t="inlineStr"/>
+      <c r="I347" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J347" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K347" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L347" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M347" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-07-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="348" ht="55" customHeight="1">
+      <c r="A348" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B348" s="123" t="inlineStr">
+        <is>
+          <t>Söker dig som gillar ett aktivt jobb, som personlig assistent i Uppsala</t>
+        </is>
+      </c>
+      <c r="C348" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D348" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E348" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F348" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G348" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H348" s="146" t="inlineStr"/>
+      <c r="I348" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J348" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K348" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L348" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M348" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="349" ht="55" customHeight="1">
+      <c r="A349" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B349" s="123" t="inlineStr">
+        <is>
+          <t>Aktiv engagerad assistent sökes till kille i Tobo/Örbyhus, körkort krav</t>
+        </is>
+      </c>
+      <c r="C349" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D349" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E349" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F349" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G349" s="146" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS</t>
+        </is>
+      </c>
+      <c r="H349" s="146" t="inlineStr"/>
+      <c r="I349" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J349" s="145" t="inlineStr">
+        <is>
+          <t>🚗 KRÄVS · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K349" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L349" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M349" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="350" ht="55" customHeight="1">
+      <c r="A350" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B350" s="123" t="inlineStr">
+        <is>
+          <t>40% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C350" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D350" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E350" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F350" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G350" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H350" s="146" t="inlineStr"/>
+      <c r="I350" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J350" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K350" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L350" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M350" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-05
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="351" ht="55" customHeight="1">
+      <c r="A351" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B351" s="123" t="inlineStr">
+        <is>
+          <t>50% tjänst erbjudes till glad kille i Almunge</t>
+        </is>
+      </c>
+      <c r="C351" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D351" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E351" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F351" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G351" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H351" s="146" t="inlineStr"/>
+      <c r="I351" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J351" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K351" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L351" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M351" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="352" ht="55" customHeight="1">
+      <c r="A352" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B352" s="123" t="inlineStr">
+        <is>
+          <t>Har du barnasinnet kvar? Då har vi rätt jobb åt dig!</t>
+        </is>
+      </c>
+      <c r="C352" s="145" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D352" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E352" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F352" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G352" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H352" s="146" t="inlineStr"/>
+      <c r="I352" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J352" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K352" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L352" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M352" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-18
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="353" ht="55" customHeight="1">
+      <c r="A353" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B353" s="123" t="inlineStr">
+        <is>
+          <t>Personlig assistent till ung man i Uppsala</t>
+        </is>
+      </c>
+      <c r="C353" s="145" t="inlineStr">
+        <is>
+          <t>A-Assistans Leimir AB</t>
+        </is>
+      </c>
+      <c r="D353" s="145" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E353" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F353" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G353" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H353" s="146" t="inlineStr"/>
+      <c r="I353" s="146" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J353" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K353" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L353" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M353" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-13
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="354" ht="55" customHeight="1">
+      <c r="A354" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B354" s="129" t="inlineStr">
+        <is>
+          <t>Söker dig personlig assistent med intresse av matlagning och omvårdnad</t>
+        </is>
+      </c>
+      <c r="C354" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D354" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E354" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F354" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G354" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H354" s="153" t="inlineStr"/>
+      <c r="I354" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J354" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K354" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L354" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M354" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-17
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="355" ht="55" customHeight="1">
+      <c r="A355" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B355" s="129" t="inlineStr">
+        <is>
+          <t>Sommaren är räddad - Vi söker dig som vill jobba!</t>
+        </is>
+      </c>
+      <c r="C355" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D355" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E355" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F355" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G355" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H355" s="153" t="inlineStr"/>
+      <c r="I355" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J355" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K355" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L355" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M355" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-04-08
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="356" ht="55" customHeight="1">
+      <c r="A356" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B356" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent- Uppsala</t>
+        </is>
+      </c>
+      <c r="C356" s="152" t="inlineStr">
+        <is>
+          <t>Inova Assistans AB</t>
+        </is>
+      </c>
+      <c r="D356" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E356" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F356" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G356" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H356" s="153" t="inlineStr"/>
+      <c r="I356" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J356" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K356" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L356" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Behovsanst.</t>
+        </is>
+      </c>
+      <c r="M356" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-31
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="357" ht="55" customHeight="1">
+      <c r="A357" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B357" s="129" t="inlineStr">
+        <is>
+          <t>Engagerad assistent sökes till man i Enköping</t>
+        </is>
+      </c>
+      <c r="C357" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D357" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E357" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F357" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G357" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H357" s="153" t="inlineStr"/>
+      <c r="I357" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J357" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · ❓</t>
+        </is>
+      </c>
+      <c r="K357" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L357" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M357" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="358" ht="55" customHeight="1">
+      <c r="A358" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B358" s="129" t="inlineStr">
+        <is>
+          <t>Sommarvik med chans till förlängning  sökes till 29årig kille i Norrtälje</t>
+        </is>
+      </c>
+      <c r="C358" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D358" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E358" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F358" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G358" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H358" s="153" t="inlineStr"/>
+      <c r="I358" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J358" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K358" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L358" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M358" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="359" ht="55" customHeight="1">
+      <c r="A359" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B359" s="129" t="inlineStr">
+        <is>
+          <t>Extra jobb nu och i sommar? Vi söker Personliga assistenter!</t>
+        </is>
+      </c>
+      <c r="C359" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D359" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E359" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F359" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G359" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H359" s="153" t="inlineStr"/>
+      <c r="I359" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J359" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K359" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L359" s="155" t="inlineStr">
+        <is>
+          <t>🔴
+Sommarvikariat.</t>
+        </is>
+      </c>
+      <c r="M359" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-30
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="360" ht="55" customHeight="1">
+      <c r="A360" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B360" s="129" t="inlineStr">
+        <is>
+          <t>Vi söker PA för kund i Stockholm</t>
+        </is>
+      </c>
+      <c r="C360" s="152" t="inlineStr">
+        <is>
+          <t>Alma Assistans AB</t>
+        </is>
+      </c>
+      <c r="D360" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E360" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F360" s="152" t="inlineStr">
+        <is>
+          <t>❓</t>
+        </is>
+      </c>
+      <c r="G360" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H360" s="153" t="inlineStr"/>
+      <c r="I360" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J360" s="152" t="inlineStr">
+        <is>
+          <t>– · ❓</t>
+        </is>
+      </c>
+      <c r="K360" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L360" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M360" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-03-23
+🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="361" ht="55" customHeight="1">
+      <c r="A361" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B361" s="129" t="inlineStr">
+        <is>
+          <t>Vill du assistera mig på min gård utanför Uppsala?</t>
+        </is>
+      </c>
+      <c r="C361" s="152" t="inlineStr">
+        <is>
+          <t>Nära AB</t>
+        </is>
+      </c>
+      <c r="D361" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E361" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F361" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G361" s="153" t="inlineStr">
+        <is>
+          <t>🚗 Merit</t>
+        </is>
+      </c>
+      <c r="H361" s="153" t="inlineStr"/>
+      <c r="I361" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J361" s="152" t="inlineStr">
+        <is>
+          <t>🚗 Merit · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K361" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L361" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Kontrollera.</t>
+        </is>
+      </c>
+      <c r="M361" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-02-19
+🟠 ledigajobbiuppsala.se</t>
         </is>
       </c>
     </row>
@@ -24174,6 +25163,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B344" r:id="rId304"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B345" r:id="rId305"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B346" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B347" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B348" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B349" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B350" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B351" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B352" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B353" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B354" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B355" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B356" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B357" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B358" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B359" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B360" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B361" r:id="rId321"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: PA-jobb uppdatering 2026-09-04
</commit_message>
<xml_diff>
--- a/PA_Jobb_Uppsala_Gunsta.xlsx
+++ b/PA_Jobb_Uppsala_Gunsta.xlsx
@@ -3102,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M361"/>
+  <dimension ref="A1:M364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3123,7 +3123,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="161" t="inlineStr">
         <is>
-          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-08-31 · 8 källor · Radie &lt;50 km · 15 nya · 1 borttagna</t>
+          <t>📋 PA-jobb Uppsala · UPPDATERAD 2026-09-04 · 8 källor · Radie &lt;50 km · 3 nya · 0 borttagna</t>
         </is>
       </c>
     </row>
@@ -24843,6 +24843,216 @@
           <t>🆕 NYTT
 2026-02-19
 🟠 ledigajobbiuppsala.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="362" ht="55" customHeight="1">
+      <c r="A362" s="144" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐⭐</t>
+        </is>
+      </c>
+      <c r="B362" s="123" t="inlineStr">
+        <is>
+          <t>19-årig kille i Knivsta söker personlig assistent - extrajobb</t>
+        </is>
+      </c>
+      <c r="C362" s="145" t="inlineStr">
+        <is>
+          <t>Vivida Assistans AB</t>
+        </is>
+      </c>
+      <c r="D362" s="145" t="inlineStr">
+        <is>
+          <t>Knivsta</t>
+        </is>
+      </c>
+      <c r="E362" s="145" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F362" s="145" t="inlineStr">
+        <is>
+          <t>✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="G362" s="146" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H362" s="146" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="I362" s="146" t="inlineStr">
+        <is>
+          <t>~27 km</t>
+        </is>
+      </c>
+      <c r="J362" s="145" t="inlineStr">
+        <is>
+          <t>– · ✅ Helg/kväll</t>
+        </is>
+      </c>
+      <c r="K362" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L362" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M362" s="149" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-03
+🏛️ Platsbanken #31435697</t>
+        </is>
+      </c>
+    </row>
+    <row r="363" ht="55" customHeight="1">
+      <c r="A363" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B363" s="129" t="inlineStr">
+        <is>
+          <t>Personlig assistent till kille i Uppsala</t>
+        </is>
+      </c>
+      <c r="C363" s="152" t="inlineStr">
+        <is>
+          <t>Inkludera Assistans AB</t>
+        </is>
+      </c>
+      <c r="D363" s="152" t="inlineStr">
+        <is>
+          <t>Uppsala</t>
+        </is>
+      </c>
+      <c r="E363" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F363" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G363" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H363" s="153" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="I363" s="153" t="inlineStr">
+        <is>
+          <t>~13 km</t>
+        </is>
+      </c>
+      <c r="J363" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K363" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L363" s="148" t="inlineStr">
+        <is>
+          <t>🟢
+Tills vidare.</t>
+        </is>
+      </c>
+      <c r="M363" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-03
+🏛️ Platsbanken #31435787</t>
+        </is>
+      </c>
+    </row>
+    <row r="364" ht="55" customHeight="1">
+      <c r="A364" s="151" t="inlineStr">
+        <is>
+          <t>🆕 ⭐⭐</t>
+        </is>
+      </c>
+      <c r="B364" s="129" t="inlineStr">
+        <is>
+          <t>Personliga assistenter sökes till man i Österbybruk – dag, kväll &amp; natt</t>
+        </is>
+      </c>
+      <c r="C364" s="152" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="D364" s="152" t="inlineStr">
+        <is>
+          <t>Östhammar</t>
+        </is>
+      </c>
+      <c r="E364" s="152" t="inlineStr">
+        <is>
+          <t>Deltid</t>
+        </is>
+      </c>
+      <c r="F364" s="152" t="inlineStr">
+        <is>
+          <t>🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="G364" s="153" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H364" s="153" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="I364" s="153" t="inlineStr">
+        <is>
+          <t>~49 km</t>
+        </is>
+      </c>
+      <c r="J364" s="152" t="inlineStr">
+        <is>
+          <t>– · 🟡 Möjligt</t>
+        </is>
+      </c>
+      <c r="K364" s="147" t="inlineStr">
+        <is>
+          <t>♂️ Man</t>
+        </is>
+      </c>
+      <c r="L364" s="159" t="inlineStr">
+        <is>
+          <t>🟡
+Diskutera semester.</t>
+        </is>
+      </c>
+      <c r="M364" s="154" t="inlineStr">
+        <is>
+          <t>🆕 NYTT
+2026-09-03
+🏛️ Platsbanken #31434238</t>
         </is>
       </c>
     </row>
@@ -25178,6 +25388,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B359" r:id="rId319"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B360" r:id="rId320"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B361" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B362" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B363" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B364" r:id="rId324"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>